<commit_message>
Re-run alternative model on the current scenarios (updates macro_scenarios.png)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables/stress_test_results.xlsx
+++ b/output/tables/stress_test_results.xlsx
@@ -152,15 +152,15 @@
     <t>BBNI</t>
   </si>
   <si>
+    <t>INPC</t>
+  </si>
+  <si>
     <t>BMRI</t>
   </si>
   <si>
     <t>BVIC</t>
   </si>
   <si>
-    <t>INPC</t>
-  </si>
-  <si>
     <t>SDRA</t>
   </si>
   <si>
@@ -182,15 +182,15 @@
     <t>BEKS</t>
   </si>
   <si>
+    <t>BSIM</t>
+  </si>
+  <si>
     <t>NISP</t>
   </si>
   <si>
     <t>BNGA</t>
   </si>
   <si>
-    <t>BSIM</t>
-  </si>
-  <si>
     <t>MEGA</t>
   </si>
   <si>
@@ -227,10 +227,10 @@
     <t>DNAR</t>
   </si>
   <si>
+    <t>BBMD</t>
+  </si>
+  <si>
     <t>BMAS</t>
-  </si>
-  <si>
-    <t>BBMD</t>
   </si>
   <si>
     <t>BBYB</t>
@@ -707,22 +707,22 @@
         <v>46</v>
       </c>
       <c r="C9" s="2">
-        <v>22.705408096313477</v>
+        <v>22.687021255493164</v>
       </c>
       <c r="D9" s="2">
-        <v>21.534833908081055</v>
+        <v>21.516447067260742</v>
       </c>
       <c r="E9" s="2">
-        <v>2.0504615306854248</v>
+        <v>2.0526115894317627</v>
       </c>
       <c r="F9" s="2">
-        <v>1.7516899108886719</v>
+        <v>1.7176399230957031</v>
       </c>
       <c r="G9" s="2">
-        <v>0.21047800779342651</v>
+        <v>0.21092790365219116</v>
       </c>
       <c r="H9" s="2">
-        <v>0.0469697006046772</v>
+        <v>0.058575522154569626</v>
       </c>
       <c r="I9" t="s">
         <v>10</v>
@@ -736,22 +736,22 @@
         <v>46</v>
       </c>
       <c r="C10" s="2">
-        <v>22.783967971801758</v>
+        <v>22.741250991821289</v>
       </c>
       <c r="D10" s="2">
-        <v>21.623571395874023</v>
+        <v>21.580854415893555</v>
       </c>
       <c r="E10" s="2">
-        <v>2.0532705783843994</v>
+        <v>2.0704705715179443</v>
       </c>
       <c r="F10" s="2">
-        <v>1.6219191551208496</v>
+        <v>1.5625275373458862</v>
       </c>
       <c r="G10" s="2">
-        <v>0.25215059518814087</v>
+        <v>0.25588491559028625</v>
       </c>
       <c r="H10" s="2">
-        <v>0.046521466225385666</v>
+        <v>0.058143459260463715</v>
       </c>
       <c r="I10" t="s">
         <v>10</v>
@@ -765,22 +765,22 @@
         <v>46</v>
       </c>
       <c r="C11" s="2">
-        <v>22.850744247436524</v>
+        <v>22.782941818237305</v>
       </c>
       <c r="D11" s="2">
-        <v>21.698825836181641</v>
+        <v>21.631023406982422</v>
       </c>
       <c r="E11" s="2">
-        <v>2.0713176727294922</v>
+        <v>2.1219062805175781</v>
       </c>
       <c r="F11" s="2">
-        <v>1.4604101181030273</v>
+        <v>1.3787004947662354</v>
       </c>
       <c r="G11" s="2">
-        <v>0.30322366952896118</v>
+        <v>0.31423038244247437</v>
       </c>
       <c r="H11" s="2">
-        <v>0.046090118587017059</v>
+        <v>0.051766075193881989</v>
       </c>
       <c r="I11" t="s">
         <v>10</v>
@@ -823,22 +823,22 @@
         <v>46</v>
       </c>
       <c r="C13" s="2">
-        <v>22.557985305786133</v>
+        <v>22.548715591430664</v>
       </c>
       <c r="D13" s="2">
-        <v>21.373861312866211</v>
+        <v>21.364589691162109</v>
       </c>
       <c r="E13" s="2">
         <v>2.0641086101531983</v>
       </c>
       <c r="F13" s="2">
-        <v>1.6760023832321167</v>
+        <v>1.6592762470245361</v>
       </c>
       <c r="G13" s="2">
         <v>0.21004875004291535</v>
       </c>
       <c r="H13" s="2">
-        <v>0.093818768858909607</v>
+        <v>0.099764458835124969</v>
       </c>
       <c r="I13" t="s">
         <v>11</v>
@@ -852,22 +852,22 @@
         <v>46</v>
       </c>
       <c r="C14" s="2">
-        <v>22.554830551147461</v>
+        <v>22.532205581665039</v>
       </c>
       <c r="D14" s="2">
-        <v>21.379356384277344</v>
+        <v>21.356731414794922</v>
       </c>
       <c r="E14" s="2">
-        <v>2.0527753829956055</v>
+        <v>2.0601809024810791</v>
       </c>
       <c r="F14" s="2">
-        <v>1.3792616128921509</v>
+        <v>1.3478525876998901</v>
       </c>
       <c r="G14" s="2">
-        <v>0.29039844870567322</v>
+        <v>0.29223448038101196</v>
       </c>
       <c r="H14" s="2">
-        <v>0.1097046434879303</v>
+        <v>0.11595332622528076</v>
       </c>
       <c r="I14" t="s">
         <v>11</v>
@@ -881,22 +881,22 @@
         <v>46</v>
       </c>
       <c r="C15" s="2">
-        <v>22.532943725585938</v>
+        <v>22.491546630859375</v>
       </c>
       <c r="D15" s="2">
-        <v>21.362756729125977</v>
+        <v>21.321361541748047</v>
       </c>
       <c r="E15" s="2">
-        <v>2.0792112350463867</v>
+        <v>2.1012980937957764</v>
       </c>
       <c r="F15" s="2">
-        <v>1.0782065391540527</v>
+        <v>1.0260818004608154</v>
       </c>
       <c r="G15" s="2">
-        <v>0.37855768203735352</v>
+        <v>0.38420450687408447</v>
       </c>
       <c r="H15" s="2">
-        <v>0.10809028893709183</v>
+        <v>0.11435664445161819</v>
       </c>
       <c r="I15" t="s">
         <v>11</v>
@@ -910,22 +910,22 @@
         <v>46</v>
       </c>
       <c r="C16" s="2">
-        <v>22.468803405761719</v>
+        <v>22.409818649291992</v>
       </c>
       <c r="D16" s="2">
-        <v>21.300548553466797</v>
+        <v>21.24156379699707</v>
       </c>
       <c r="E16" s="2">
-        <v>2.1561546325683594</v>
+        <v>2.1993710994720459</v>
       </c>
       <c r="F16" s="2">
-        <v>0.69931495189666748</v>
+        <v>0.63403975963592529</v>
       </c>
       <c r="G16" s="2">
-        <v>0.4889063835144043</v>
+        <v>0.50107765197753906</v>
       </c>
       <c r="H16" s="2">
-        <v>0.10659576952457428</v>
+        <v>0.10688376426696777</v>
       </c>
       <c r="I16" t="s">
         <v>11</v>
@@ -1060,7 +1060,7 @@
         <v>22.532503128051758</v>
       </c>
       <c r="C3" s="2">
-        <v>22.850744247436524</v>
+        <v>22.782941818237305</v>
       </c>
       <c r="D3" s="2">
         <v>22.532503128051758</v>
@@ -1069,28 +1069,28 @@
         <v>21.336328506469727</v>
       </c>
       <c r="F3" s="2">
-        <v>21.698825836181641</v>
+        <v>21.631023406982422</v>
       </c>
       <c r="G3" s="2">
         <v>2.0984182357788086</v>
       </c>
       <c r="H3" s="2">
-        <v>2.0713176727294922</v>
+        <v>2.1219062805175781</v>
       </c>
       <c r="I3" s="2">
-        <v>7.1552333831787109</v>
+        <v>7.272301197052002</v>
       </c>
       <c r="J3" s="2">
-        <v>2.7096412181854248</v>
+        <v>2.746051549911499</v>
       </c>
       <c r="K3" s="2">
-        <v>1.3792003393173218</v>
+        <v>1.6003671884536743</v>
       </c>
       <c r="L3" s="2">
-        <v>12.804572105407715</v>
+        <v>12.468243598937988</v>
       </c>
       <c r="M3" s="2">
-        <v>83.839576721191406</v>
+        <v>81.96295166015625</v>
       </c>
       <c r="N3" s="2">
         <v>1</v>
@@ -1116,37 +1116,37 @@
         <v>22.532503128051758</v>
       </c>
       <c r="C4" s="2">
-        <v>22.468803405761719</v>
+        <v>22.409818649291992</v>
       </c>
       <c r="D4" s="2">
-        <v>22.468803405761719</v>
+        <v>22.409818649291992</v>
       </c>
       <c r="E4" s="2">
         <v>21.336328506469727</v>
       </c>
       <c r="F4" s="2">
-        <v>21.300548553466797</v>
+        <v>21.24156379699707</v>
       </c>
       <c r="G4" s="2">
         <v>2.0984182357788086</v>
       </c>
       <c r="H4" s="2">
-        <v>2.1561546325683594</v>
+        <v>2.1993710994720459</v>
       </c>
       <c r="I4" s="2">
-        <v>10.37814998626709</v>
+        <v>10.527677536010742</v>
       </c>
       <c r="J4" s="2">
-        <v>5.8325252532958984</v>
+        <v>5.9048905372619629</v>
       </c>
       <c r="K4" s="2">
-        <v>3.1689927577972412</v>
+        <v>3.3108038902282715</v>
       </c>
       <c r="L4" s="2">
-        <v>9.1392679214477539</v>
+        <v>8.8250494003295898</v>
       </c>
       <c r="M4" s="2">
-        <v>76.607666015625</v>
+        <v>76.075386047363281</v>
       </c>
       <c r="N4" s="2">
         <v>3</v>
@@ -1416,22 +1416,22 @@
         <v>46296</v>
       </c>
       <c r="D9" s="2">
-        <v>32.293148040771484</v>
+        <v>32.196323394775391</v>
       </c>
       <c r="E9" s="2">
-        <v>30.994831085205078</v>
+        <v>30.898006439208984</v>
       </c>
       <c r="F9" s="2">
-        <v>2.3390774726867676</v>
+        <v>2.3415219783782959</v>
       </c>
       <c r="G9" s="2">
-        <v>0.099569372832775116</v>
+        <v>0.05543874204158783</v>
       </c>
       <c r="H9" s="2">
-        <v>0.32255697250366211</v>
+        <v>0.32286614179611206</v>
       </c>
       <c r="I9" s="2">
-        <v>0.21919785439968109</v>
+        <v>0.27335980534553528</v>
       </c>
     </row>
     <row r="10">
@@ -1445,22 +1445,22 @@
         <v>46388</v>
       </c>
       <c r="D10" s="2">
-        <v>31.551193237304688</v>
+        <v>31.347814559936524</v>
       </c>
       <c r="E10" s="2">
-        <v>30.264167785644531</v>
+        <v>30.060787200927734</v>
       </c>
       <c r="F10" s="2">
-        <v>2.3382308483123779</v>
+        <v>2.3577568531036377</v>
       </c>
       <c r="G10" s="2">
-        <v>-0.04799332469701767</v>
+        <v>-0.1241750568151474</v>
       </c>
       <c r="H10" s="2">
-        <v>0.36602482199668884</v>
+        <v>0.36874857544898987</v>
       </c>
       <c r="I10" s="2">
-        <v>0.21710602939128876</v>
+        <v>0.27134346961975098</v>
       </c>
     </row>
     <row r="11">
@@ -1474,22 +1474,22 @@
         <v>46478</v>
       </c>
       <c r="D11" s="2">
-        <v>30.793735504150391</v>
+        <v>30.52039909362793</v>
       </c>
       <c r="E11" s="2">
-        <v>29.516111373901367</v>
+        <v>29.242774963378906</v>
       </c>
       <c r="F11" s="2">
-        <v>2.3612833023071289</v>
+        <v>2.4187808036804199</v>
       </c>
       <c r="G11" s="2">
-        <v>-0.2319815456867218</v>
+        <v>-0.32962366938591003</v>
       </c>
       <c r="H11" s="2">
-        <v>0.41871011257171631</v>
+        <v>0.42734315991401672</v>
       </c>
       <c r="I11" s="2">
-        <v>0.21509301662445068</v>
+        <v>0.24158152937889099</v>
       </c>
     </row>
     <row r="12">
@@ -1532,22 +1532,22 @@
         <v>46204</v>
       </c>
       <c r="D13" s="2">
-        <v>32.627864837646484</v>
+        <v>32.577632904052734</v>
       </c>
       <c r="E13" s="2">
-        <v>31.314519882202149</v>
+        <v>31.264287948608398</v>
       </c>
       <c r="F13" s="2">
         <v>2.3676373958587647</v>
       </c>
       <c r="G13" s="2">
-        <v>0.016034509986639023</v>
+        <v>-0.0066980868577957153</v>
       </c>
       <c r="H13" s="2">
         <v>0.32043734192848206</v>
       </c>
       <c r="I13" s="2">
-        <v>0.43783271312713623</v>
+        <v>0.46558001637458801</v>
       </c>
     </row>
     <row r="14">
@@ -1561,22 +1561,22 @@
         <v>46296</v>
       </c>
       <c r="D14" s="2">
-        <v>31.383514404296875</v>
+        <v>31.275106430053711</v>
       </c>
       <c r="E14" s="2">
-        <v>30.079765319824219</v>
+        <v>29.971355438232422</v>
       </c>
       <c r="F14" s="2">
-        <v>2.3417079448699951</v>
+        <v>2.3501265048980713</v>
       </c>
       <c r="G14" s="2">
-        <v>-0.32482168078422546</v>
+        <v>-0.365724116563797</v>
       </c>
       <c r="H14" s="2">
-        <v>0.40269258618354797</v>
+        <v>0.40404412150382996</v>
       </c>
       <c r="I14" s="2">
-        <v>0.51196885108947754</v>
+        <v>0.54113012552261353</v>
       </c>
     </row>
     <row r="15">
@@ -1590,22 +1590,22 @@
         <v>46388</v>
       </c>
       <c r="D15" s="2">
-        <v>30.119583129882813</v>
+        <v>29.939483642578125</v>
       </c>
       <c r="E15" s="2">
-        <v>28.821697235107422</v>
+        <v>28.641597747802734</v>
       </c>
       <c r="F15" s="2">
-        <v>2.3676788806915283</v>
+        <v>2.3927505016326904</v>
       </c>
       <c r="G15" s="2">
-        <v>-0.6657598614692688</v>
+        <v>-0.73529845476150513</v>
       </c>
       <c r="H15" s="2">
-        <v>0.49121877551078796</v>
+        <v>0.49572631716728211</v>
       </c>
       <c r="I15" s="2">
-        <v>0.50443494319915771</v>
+        <v>0.53367871046066284</v>
       </c>
     </row>
     <row r="16">
@@ -1619,22 +1619,22 @@
         <v>46478</v>
       </c>
       <c r="D16" s="2">
-        <v>28.787729263305664</v>
+        <v>28.573301315307617</v>
       </c>
       <c r="E16" s="2">
-        <v>27.491985321044922</v>
+        <v>27.277557373046875</v>
       </c>
       <c r="F16" s="2">
-        <v>2.4577007293701172</v>
+        <v>2.5068068504333496</v>
       </c>
       <c r="G16" s="2">
-        <v>-1.0960925817489624</v>
+        <v>-1.1780779361724854</v>
       </c>
       <c r="H16" s="2">
-        <v>0.60087126493453979</v>
+        <v>0.61131542921066284</v>
       </c>
       <c r="I16" s="2">
-        <v>0.49746036529541016</v>
+        <v>0.49880436062812805</v>
       </c>
     </row>
     <row r="17">
@@ -1851,22 +1851,22 @@
         <v>46296</v>
       </c>
       <c r="D24" s="2">
-        <v>19.855304718017578</v>
+        <v>19.791816711425781</v>
       </c>
       <c r="E24" s="2">
-        <v>18.338617324829102</v>
+        <v>18.275131225585938</v>
       </c>
       <c r="F24" s="2">
-        <v>5.1348214149475098</v>
+        <v>5.1400241851806641</v>
       </c>
       <c r="G24" s="2">
-        <v>-0.5272565484046936</v>
+        <v>-0.59366512298583984</v>
       </c>
       <c r="H24" s="2">
-        <v>0.44036611914634705</v>
+        <v>0.44137194752693176</v>
       </c>
       <c r="I24" s="2">
-        <v>0.10887981951236725</v>
+        <v>0.13578310608863831</v>
       </c>
     </row>
     <row r="25">
@@ -1880,22 +1880,22 @@
         <v>46388</v>
       </c>
       <c r="D25" s="2">
-        <v>19.045539855957031</v>
+        <v>18.8912353515625</v>
       </c>
       <c r="E25" s="2">
-        <v>17.542041778564453</v>
+        <v>17.387737274169922</v>
       </c>
       <c r="F25" s="2">
-        <v>5.4094581604003906</v>
+        <v>5.4531121253967285</v>
       </c>
       <c r="G25" s="2">
-        <v>-1.0064841508865357</v>
+        <v>-1.1398345232009888</v>
       </c>
       <c r="H25" s="2">
-        <v>0.56890207529067993</v>
+        <v>0.57767343521118164</v>
       </c>
       <c r="I25" s="2">
-        <v>0.10784076899290085</v>
+        <v>0.13478155434131622</v>
       </c>
     </row>
     <row r="26">
@@ -1909,22 +1909,22 @@
         <v>46478</v>
       </c>
       <c r="D26" s="2">
-        <v>18.024801254272461</v>
+        <v>17.767337799072266</v>
       </c>
       <c r="E26" s="2">
-        <v>16.53228759765625</v>
+        <v>16.274824142456055</v>
       </c>
       <c r="F26" s="2">
-        <v>5.7176103591918945</v>
+        <v>5.8516373634338379</v>
       </c>
       <c r="G26" s="2">
-        <v>-1.6105465888977051</v>
+        <v>-1.8204857110977173</v>
       </c>
       <c r="H26" s="2">
-        <v>0.72956866025924683</v>
+        <v>0.75692063570022583</v>
       </c>
       <c r="I26" s="2">
-        <v>0.10684086382389069</v>
+        <v>0.11999822407960892</v>
       </c>
     </row>
     <row r="27">
@@ -1967,22 +1967,22 @@
         <v>46204</v>
       </c>
       <c r="D28" s="2">
-        <v>20.198644638061523</v>
+        <v>20.166908264160156</v>
       </c>
       <c r="E28" s="2">
-        <v>18.664400100708008</v>
+        <v>18.632665634155274</v>
       </c>
       <c r="F28" s="2">
         <v>4.8930139541625977</v>
       </c>
       <c r="G28" s="2">
-        <v>-0.53119397163391113</v>
+        <v>-0.56323736906051636</v>
       </c>
       <c r="H28" s="2">
         <v>0.41087499260902405</v>
       </c>
       <c r="I28" s="2">
-        <v>0.21747998893260956</v>
+        <v>0.23126260936260223</v>
       </c>
     </row>
     <row r="29">
@@ -1996,22 +1996,22 @@
         <v>46296</v>
       </c>
       <c r="D29" s="2">
-        <v>19.060317993164063</v>
+        <v>18.981084823608399</v>
       </c>
       <c r="E29" s="2">
-        <v>17.537282943725586</v>
+        <v>17.458049774169922</v>
       </c>
       <c r="F29" s="2">
-        <v>5.1404204368591309</v>
+        <v>5.1583356857299805</v>
       </c>
       <c r="G29" s="2">
-        <v>-1.4064042568206787</v>
+        <v>-1.4747363328933716</v>
       </c>
       <c r="H29" s="2">
-        <v>0.62382179498672485</v>
+        <v>0.62792086601257324</v>
       </c>
       <c r="I29" s="2">
-        <v>0.25430482625961304</v>
+        <v>0.26878979802131653</v>
       </c>
     </row>
     <row r="30">
@@ -2025,22 +2025,22 @@
         <v>46388</v>
       </c>
       <c r="D30" s="2">
-        <v>17.577241897583008</v>
+        <v>17.423500061035156</v>
       </c>
       <c r="E30" s="2">
-        <v>16.061058044433594</v>
+        <v>15.907316207885742</v>
       </c>
       <c r="F30" s="2">
-        <v>5.475285530090332</v>
+        <v>5.5312871932983398</v>
       </c>
       <c r="G30" s="2">
-        <v>-2.3986327648162842</v>
+        <v>-2.5258476734161377</v>
       </c>
       <c r="H30" s="2">
-        <v>0.87370198965072632</v>
+        <v>0.8869701623916626</v>
       </c>
       <c r="I30" s="2">
-        <v>0.25056260824203491</v>
+        <v>0.26508855819702148</v>
       </c>
     </row>
     <row r="31">
@@ -2054,22 +2054,22 @@
         <v>46478</v>
       </c>
       <c r="D31" s="2">
-        <v>15.59735107421875</v>
+        <v>15.363493919372559</v>
       </c>
       <c r="E31" s="2">
-        <v>14.08366870880127</v>
+        <v>13.849811553955078</v>
       </c>
       <c r="F31" s="2">
-        <v>5.9422268867492676</v>
+        <v>6.0563716888427734</v>
       </c>
       <c r="G31" s="2">
-        <v>-3.7030303478240967</v>
+        <v>-3.8843579292297363</v>
       </c>
       <c r="H31" s="2">
-        <v>1.1976770162582397</v>
+        <v>1.2274543046951294</v>
       </c>
       <c r="I31" s="2">
-        <v>0.24709819257259369</v>
+        <v>0.24776577949523926</v>
       </c>
     </row>
     <row r="32">
@@ -2286,22 +2286,22 @@
         <v>46296</v>
       </c>
       <c r="D39" s="2">
-        <v>25.061229705810547</v>
+        <v>25.040300369262695</v>
       </c>
       <c r="E39" s="2">
-        <v>23.808938980102539</v>
+        <v>23.788009643554688</v>
       </c>
       <c r="F39" s="2">
-        <v>1.9204545021057129</v>
+        <v>1.9224815368652344</v>
       </c>
       <c r="G39" s="2">
-        <v>1.1512627601623535</v>
+        <v>1.1219563484191895</v>
       </c>
       <c r="H39" s="2">
-        <v>0.21882490813732147</v>
+        <v>0.21925754845142365</v>
       </c>
       <c r="I39" s="2">
-        <v>0.057834040373563766</v>
+        <v>0.07212434709072113</v>
       </c>
     </row>
     <row r="40">
@@ -2315,22 +2315,22 @@
         <v>46388</v>
       </c>
       <c r="D40" s="2">
-        <v>25.010759353637695</v>
+        <v>24.966054916381836</v>
       </c>
       <c r="E40" s="2">
-        <v>23.769357681274414</v>
+        <v>23.724653244018555</v>
       </c>
       <c r="F40" s="2">
-        <v>1.90349280834198</v>
+        <v>1.919559121131897</v>
       </c>
       <c r="G40" s="2">
-        <v>1.0417324304580688</v>
+        <v>0.99419897794723511</v>
       </c>
       <c r="H40" s="2">
-        <v>0.25532576441764832</v>
+        <v>0.25887519121170044</v>
       </c>
       <c r="I40" s="2">
-        <v>0.057282127439975739</v>
+        <v>0.071592345833778381</v>
       </c>
     </row>
     <row r="41">
@@ -2344,22 +2344,22 @@
         <v>46478</v>
       </c>
       <c r="D41" s="2">
-        <v>24.963764190673828</v>
+        <v>24.897043228149414</v>
       </c>
       <c r="E41" s="2">
-        <v>23.73143196105957</v>
+        <v>23.664709091186524</v>
       </c>
       <c r="F41" s="2">
-        <v>1.9009175300598145</v>
+        <v>1.9477556943893433</v>
       </c>
       <c r="G41" s="2">
-        <v>0.90587246417999268</v>
+        <v>0.83984202146530151</v>
       </c>
       <c r="H41" s="2">
-        <v>0.29969987273216248</v>
+        <v>0.31015285849571228</v>
       </c>
       <c r="I41" s="2">
-        <v>0.056751005351543427</v>
+        <v>0.063739843666553497</v>
       </c>
     </row>
     <row r="42">
@@ -2402,22 +2402,22 @@
         <v>46204</v>
       </c>
       <c r="D43" s="2">
-        <v>25.047008514404297</v>
+        <v>25.036436080932617</v>
       </c>
       <c r="E43" s="2">
-        <v>23.780221939086914</v>
+        <v>23.769649505615234</v>
       </c>
       <c r="F43" s="2">
         <v>1.9531245231628418</v>
       </c>
       <c r="G43" s="2">
-        <v>1.0657336711883545</v>
+        <v>1.0514113903045654</v>
       </c>
       <c r="H43" s="2">
         <v>0.22081294655799866</v>
       </c>
       <c r="I43" s="2">
-        <v>0.11551954597234726</v>
+        <v>0.12284050136804581</v>
       </c>
     </row>
     <row r="44">
@@ -2431,22 +2431,22 @@
         <v>46296</v>
       </c>
       <c r="D44" s="2">
-        <v>24.891687393188477</v>
+        <v>24.866565704345703</v>
       </c>
       <c r="E44" s="2">
-        <v>23.6341552734375</v>
+        <v>23.609031677246094</v>
       </c>
       <c r="F44" s="2">
-        <v>1.9226356744766235</v>
+        <v>1.9296172857284546</v>
       </c>
       <c r="G44" s="2">
-        <v>0.79852628707885742</v>
+        <v>0.77209866046905518</v>
       </c>
       <c r="H44" s="2">
-        <v>0.29408100247383118</v>
+        <v>0.2958427369594574</v>
       </c>
       <c r="I44" s="2">
-        <v>0.13507990539073944</v>
+        <v>0.14277394115924835</v>
       </c>
     </row>
     <row r="45">
@@ -2460,22 +2460,22 @@
         <v>46388</v>
       </c>
       <c r="D45" s="2">
-        <v>24.727682113647461</v>
+        <v>24.685161590576172</v>
       </c>
       <c r="E45" s="2">
-        <v>23.475805282592774</v>
+        <v>23.433286666870117</v>
       </c>
       <c r="F45" s="2">
-        <v>1.9277242422103882</v>
+        <v>1.9483597278594971</v>
       </c>
       <c r="G45" s="2">
-        <v>0.5266912579536438</v>
+        <v>0.48454341292381287</v>
       </c>
       <c r="H45" s="2">
-        <v>0.37324488162994385</v>
+        <v>0.37859264016151428</v>
       </c>
       <c r="I45" s="2">
-        <v>0.13309215009212494</v>
+        <v>0.14080794155597687</v>
       </c>
     </row>
     <row r="46">
@@ -2489,22 +2489,22 @@
         <v>46478</v>
       </c>
       <c r="D46" s="2">
-        <v>24.531883239746094</v>
+        <v>24.475330352783203</v>
       </c>
       <c r="E46" s="2">
-        <v>23.282073974609375</v>
+        <v>23.225521087646484</v>
       </c>
       <c r="F46" s="2">
-        <v>1.9794753789901733</v>
+        <v>2.0195136070251465</v>
       </c>
       <c r="G46" s="2">
-        <v>0.18676139414310455</v>
+        <v>0.13338294625282288</v>
       </c>
       <c r="H46" s="2">
-        <v>0.47149252891540527</v>
+        <v>0.48288843035697937</v>
       </c>
       <c r="I46" s="2">
-        <v>0.13125194609165192</v>
+        <v>0.13160654902458191</v>
       </c>
     </row>
     <row r="47">
@@ -2721,22 +2721,22 @@
         <v>46296</v>
       </c>
       <c r="D54" s="2">
-        <v>21.514488220214844</v>
+        <v>21.506404876708984</v>
       </c>
       <c r="E54" s="2">
-        <v>20.416217803955078</v>
+        <v>20.408134460449219</v>
       </c>
       <c r="F54" s="2">
-        <v>1.7962017059326172</v>
+        <v>1.7980976104736328</v>
       </c>
       <c r="G54" s="2">
-        <v>2.3298697471618652</v>
+        <v>2.297968864440918</v>
       </c>
       <c r="H54" s="2">
-        <v>0.17613174021244049</v>
+        <v>0.1765400618314743</v>
       </c>
       <c r="I54" s="2">
-        <v>0.025086788460612297</v>
+        <v>0.031285524368286133</v>
       </c>
     </row>
     <row r="55">
@@ -2750,22 +2750,22 @@
         <v>46388</v>
       </c>
       <c r="D55" s="2">
-        <v>21.779720306396484</v>
+        <v>21.758813858032227</v>
       </c>
       <c r="E55" s="2">
-        <v>20.690998077392578</v>
+        <v>20.67009162902832</v>
       </c>
       <c r="F55" s="2">
-        <v>1.7814713716506958</v>
+        <v>1.7965060472488403</v>
       </c>
       <c r="G55" s="2">
-        <v>2.2294831275939942</v>
+        <v>2.1741983890533447</v>
       </c>
       <c r="H55" s="2">
-        <v>0.21072673797607422</v>
+        <v>0.2140783816576004</v>
       </c>
       <c r="I55" s="2">
-        <v>0.024847384542226791</v>
+        <v>0.031054757535457611</v>
       </c>
     </row>
     <row r="56">
@@ -2779,22 +2779,22 @@
         <v>46478</v>
       </c>
       <c r="D56" s="2">
-        <v>22.047395706176758</v>
+        <v>22.010776519775391</v>
       </c>
       <c r="E56" s="2">
-        <v>20.966629028320313</v>
+        <v>20.930007934570313</v>
       </c>
       <c r="F56" s="2">
-        <v>1.7801098823547363</v>
+        <v>1.8239618539810181</v>
       </c>
       <c r="G56" s="2">
-        <v>2.1051764488220215</v>
+        <v>2.0316357612609863</v>
       </c>
       <c r="H56" s="2">
-        <v>0.2529807984828949</v>
+        <v>0.26266857981681824</v>
       </c>
       <c r="I56" s="2">
-        <v>0.024616997689008713</v>
+        <v>0.027648560702800751</v>
       </c>
     </row>
     <row r="57">
@@ -2837,22 +2837,22 @@
         <v>46204</v>
       </c>
       <c r="D58" s="2">
-        <v>21.239255905151367</v>
+        <v>21.235248565673828</v>
       </c>
       <c r="E58" s="2">
-        <v>20.128271102905274</v>
+        <v>20.124263763427734</v>
       </c>
       <c r="F58" s="2">
         <v>1.8255102634429932</v>
       </c>
       <c r="G58" s="2">
-        <v>2.2511222362518311</v>
+        <v>2.2354321479797363</v>
       </c>
       <c r="H58" s="2">
         <v>0.17787288129329681</v>
       </c>
       <c r="I58" s="2">
-        <v>0.050109144300222397</v>
+        <v>0.053284771740436554</v>
       </c>
     </row>
     <row r="59">
@@ -2866,22 +2866,22 @@
         <v>46296</v>
       </c>
       <c r="D59" s="2">
-        <v>21.482038497924805</v>
+        <v>21.471294403076172</v>
       </c>
       <c r="E59" s="2">
-        <v>20.379169464111328</v>
+        <v>20.368425369262695</v>
       </c>
       <c r="F59" s="2">
-        <v>1.7982420921325684</v>
+        <v>1.8047720193862915</v>
       </c>
       <c r="G59" s="2">
-        <v>2.0055313110351563</v>
+        <v>1.9766120910644531</v>
       </c>
       <c r="H59" s="2">
-        <v>0.24715523421764374</v>
+        <v>0.24881789088249207</v>
       </c>
       <c r="I59" s="2">
-        <v>0.058593884110450745</v>
+        <v>0.061931338161230087</v>
       </c>
     </row>
     <row r="60">
@@ -2895,22 +2895,22 @@
         <v>46388</v>
       </c>
       <c r="D60" s="2">
-        <v>21.734552383422852</v>
+        <v>21.713344573974609</v>
       </c>
       <c r="E60" s="2">
-        <v>20.636646270751953</v>
+        <v>20.615438461303711</v>
       </c>
       <c r="F60" s="2">
-        <v>1.8041472434997559</v>
+        <v>1.8234575986862183</v>
       </c>
       <c r="G60" s="2">
-        <v>1.767127275466919</v>
+        <v>1.7200025320053101</v>
       </c>
       <c r="H60" s="2">
-        <v>0.322083979845047</v>
+        <v>0.32713389396667481</v>
       </c>
       <c r="I60" s="2">
-        <v>0.057731647044420242</v>
+        <v>0.061078540980815887</v>
       </c>
     </row>
     <row r="61">
@@ -2924,22 +2924,22 @@
         <v>46478</v>
       </c>
       <c r="D61" s="2">
-        <v>21.98735237121582</v>
+        <v>21.954456329345703</v>
       </c>
       <c r="E61" s="2">
-        <v>20.891258239746094</v>
+        <v>20.858362197875977</v>
       </c>
       <c r="F61" s="2">
-        <v>1.8536592721939087</v>
+        <v>1.8911439180374146</v>
       </c>
       <c r="G61" s="2">
-        <v>1.4720641374588013</v>
+        <v>1.4152282476425171</v>
       </c>
       <c r="H61" s="2">
-        <v>0.4151182770729065</v>
+        <v>0.42588469386100769</v>
       </c>
       <c r="I61" s="2">
-        <v>0.056933414191007614</v>
+        <v>0.057087235152721405</v>
       </c>
     </row>
   </sheetData>
@@ -3033,22 +3033,22 @@
         <v>13.444534301757813</v>
       </c>
       <c r="E2" s="2">
-        <v>7.997016429901123</v>
+        <v>7.0417094230651855</v>
       </c>
       <c r="F2" s="2">
-        <v>1.9058444499969482</v>
+        <v>1.1889625787734985</v>
       </c>
       <c r="G2" s="2">
-        <v>1.9058444499969482</v>
+        <v>1.1889625787734985</v>
       </c>
       <c r="H2" s="2">
         <v>3.5872464179992676</v>
       </c>
       <c r="I2" s="2">
-        <v>3.5965628623962402</v>
+        <v>3.6837797164916992</v>
       </c>
       <c r="J2" s="2">
-        <v>3.7428078651428223</v>
+        <v>3.8172707557678223</v>
       </c>
       <c r="K2" s="2">
         <v>0</v>
@@ -3066,22 +3066,22 @@
         <v>1</v>
       </c>
       <c r="P2" s="2">
-        <v>21.779239654541016</v>
+        <v>22.028060913085938</v>
       </c>
       <c r="Q2" s="2">
-        <v>24.939676284790039</v>
+        <v>28.938970565795898</v>
       </c>
       <c r="R2" s="2">
-        <v>7.997016429901123</v>
+        <v>7.0417094230651855</v>
       </c>
       <c r="S2" s="2">
         <v>1</v>
       </c>
       <c r="T2" s="2">
-        <v>28.659156799316406</v>
+        <v>28.97459602355957</v>
       </c>
       <c r="U2" s="2">
-        <v>57.303966522216797</v>
+        <v>59.868293762207031</v>
       </c>
       <c r="V2" s="2">
         <v>0</v>
@@ -3101,22 +3101,22 @@
         <v>14.296926498413086</v>
       </c>
       <c r="E3" s="2">
-        <v>9.0769309997558594</v>
+        <v>8.385279655456543</v>
       </c>
       <c r="F3" s="2">
-        <v>3.4344329833984375</v>
+        <v>2.9253649711608887</v>
       </c>
       <c r="G3" s="2">
-        <v>3.4344329833984375</v>
+        <v>2.9253649711608887</v>
       </c>
       <c r="H3" s="2">
         <v>4.3195414543151855</v>
       </c>
       <c r="I3" s="2">
-        <v>4.3306727409362793</v>
+        <v>4.4348745346069336</v>
       </c>
       <c r="J3" s="2">
-        <v>4.505373477935791</v>
+        <v>4.5942845344543457</v>
       </c>
       <c r="K3" s="2">
         <v>0</v>
@@ -3134,22 +3134,22 @@
         <v>0</v>
       </c>
       <c r="P3" s="2">
-        <v>17.868358612060547</v>
+        <v>18.252490997314453</v>
       </c>
       <c r="Q3" s="2">
-        <v>23.049930572509766</v>
+        <v>26.746189117431641</v>
       </c>
       <c r="R3" s="2">
-        <v>9.0769309997558594</v>
+        <v>8.385279655456543</v>
       </c>
       <c r="S3" s="2">
         <v>1</v>
       </c>
       <c r="T3" s="2">
-        <v>27.667943954467773</v>
+        <v>28.14610481262207</v>
       </c>
       <c r="U3" s="2">
-        <v>52.961891174316406</v>
+        <v>55.331912994384766</v>
       </c>
       <c r="V3" s="2">
         <v>0</v>
@@ -3169,22 +3169,22 @@
         <v>14.114684104919434</v>
       </c>
       <c r="E4" s="2">
-        <v>11.191521644592285</v>
+        <v>10.987530708312988</v>
       </c>
       <c r="F4" s="2">
-        <v>7.7347092628479004</v>
+        <v>7.5367732048034668</v>
       </c>
       <c r="G4" s="2">
-        <v>7.7347092628479004</v>
+        <v>7.5367732048034668</v>
       </c>
       <c r="H4" s="2">
         <v>9.4293003082275391</v>
       </c>
       <c r="I4" s="2">
-        <v>9.452301025390625</v>
+        <v>9.6672811508178711</v>
       </c>
       <c r="J4" s="2">
-        <v>9.8124170303344727</v>
+        <v>9.9950971603393555</v>
       </c>
       <c r="K4" s="2">
         <v>0</v>
@@ -3202,22 +3202,22 @@
         <v>0</v>
       </c>
       <c r="P4" s="2">
-        <v>22.204170227050781</v>
+        <v>22.800189971923828</v>
       </c>
       <c r="Q4" s="2">
-        <v>3.3274757862091065</v>
+        <v>3.8610653877258301</v>
       </c>
       <c r="R4" s="2">
-        <v>11.191521644592285</v>
+        <v>10.987530708312988</v>
       </c>
       <c r="S4" s="2">
         <v>1</v>
       </c>
       <c r="T4" s="2">
-        <v>39.587791442871094</v>
+        <v>40.338081359863281</v>
       </c>
       <c r="U4" s="2">
-        <v>7.6455507278442383</v>
+        <v>7.9876861572265625</v>
       </c>
       <c r="V4" s="2">
         <v>0</v>
@@ -3237,22 +3237,22 @@
         <v>10.378665924072266</v>
       </c>
       <c r="E5" s="2">
-        <v>9.6848545074462891</v>
+        <v>9.4984655380249024</v>
       </c>
       <c r="F5" s="2">
-        <v>8.6215848922729492</v>
+        <v>8.4442358016967773</v>
       </c>
       <c r="G5" s="2">
-        <v>8.6215848922729492</v>
+        <v>8.4442358016967773</v>
       </c>
       <c r="H5" s="2">
         <v>4.5805325508117676</v>
       </c>
       <c r="I5" s="2">
-        <v>4.5923056602478027</v>
+        <v>4.7024917602539063</v>
       </c>
       <c r="J5" s="2">
-        <v>4.7770328521728516</v>
+        <v>4.8710322380065918</v>
       </c>
       <c r="K5" s="2">
         <v>0</v>
@@ -3270,19 +3270,19 @@
         <v>0</v>
       </c>
       <c r="P5" s="2">
-        <v>13.169404029846191</v>
+        <v>13.525614738464355</v>
       </c>
       <c r="Q5" s="2">
         <v>0</v>
       </c>
       <c r="R5" s="2">
-        <v>9.6848545074462891</v>
+        <v>9.4984655380249024</v>
       </c>
       <c r="S5" s="2">
         <v>0</v>
       </c>
       <c r="T5" s="2">
-        <v>22.775430679321289</v>
+        <v>23.222873687744141</v>
       </c>
       <c r="U5" s="2">
         <v>0</v>
@@ -3305,22 +3305,22 @@
         <v>18.346424102783203</v>
       </c>
       <c r="E6" s="2">
-        <v>14.295330047607422</v>
+        <v>13.879581451416016</v>
       </c>
       <c r="F6" s="2">
-        <v>9.3762702941894531</v>
+        <v>9.0250692367553711</v>
       </c>
       <c r="G6" s="2">
-        <v>9.3762702941894531</v>
+        <v>9.0250692367553711</v>
       </c>
       <c r="H6" s="2">
         <v>7.7831716537475586</v>
       </c>
       <c r="I6" s="2">
-        <v>7.8025031089782715</v>
+        <v>7.9832682609558106</v>
       </c>
       <c r="J6" s="2">
-        <v>8.1053905487060547</v>
+        <v>8.2592029571533203</v>
       </c>
       <c r="K6" s="2">
         <v>0</v>
@@ -3338,22 +3338,22 @@
         <v>0</v>
       </c>
       <c r="P6" s="2">
-        <v>32.636619567871094</v>
+        <v>33.260562896728516</v>
       </c>
       <c r="Q6" s="2">
-        <v>8.5850620269775391</v>
+        <v>9.9617509841918945</v>
       </c>
       <c r="R6" s="2">
-        <v>14.295330047607422</v>
+        <v>13.879581451416016</v>
       </c>
       <c r="S6" s="2">
         <v>0</v>
       </c>
       <c r="T6" s="2">
-        <v>49.200946807861328</v>
+        <v>49.977306365966797</v>
       </c>
       <c r="U6" s="2">
-        <v>19.725919723510742</v>
+        <v>20.608646392822266</v>
       </c>
       <c r="V6" s="2">
         <v>0</v>
@@ -3373,22 +3373,22 @@
         <v>25.037126541137695</v>
       </c>
       <c r="E7" s="2">
-        <v>19.098236083984375</v>
+        <v>18.26716423034668</v>
       </c>
       <c r="F7" s="2">
-        <v>13.041565895080566</v>
+        <v>12.482504844665527</v>
       </c>
       <c r="G7" s="2">
-        <v>13.041565895080566</v>
+        <v>12.482504844665527</v>
       </c>
       <c r="H7" s="2">
         <v>0.43604627251625061</v>
       </c>
       <c r="I7" s="2">
-        <v>0.43721580505371094</v>
+        <v>0.44817462563514709</v>
       </c>
       <c r="J7" s="2">
-        <v>0.45560121536254883</v>
+        <v>0.46498125791549683</v>
       </c>
       <c r="K7" s="2">
         <v>0</v>
@@ -3406,22 +3406,22 @@
         <v>0</v>
       </c>
       <c r="P7" s="2">
-        <v>1.0422648191452026</v>
+        <v>1.0714079141616821</v>
       </c>
       <c r="Q7" s="2">
-        <v>21.105220794677734</v>
+        <v>24.489627838134766</v>
       </c>
       <c r="R7" s="2">
-        <v>19.098236083984375</v>
+        <v>18.26716423034668</v>
       </c>
       <c r="S7" s="2">
         <v>0</v>
       </c>
       <c r="T7" s="2">
-        <v>1.8421493768692017</v>
+        <v>1.8792433738708496</v>
       </c>
       <c r="U7" s="2">
-        <v>48.4935302734375</v>
+        <v>50.663597106933594</v>
       </c>
       <c r="V7" s="2">
         <v>0</v>
@@ -3441,22 +3441,22 @@
         <v>16.574180603027344</v>
       </c>
       <c r="E8" s="2">
-        <v>16.114725112915039</v>
+        <v>16.557954788208008</v>
       </c>
       <c r="F8" s="2">
-        <v>16.127792358398438</v>
+        <v>16.503911972045898</v>
       </c>
       <c r="G8" s="2">
-        <v>16.127792358398438</v>
+        <v>16.503911972045898</v>
       </c>
       <c r="H8" s="2">
         <v>2.2926928997039795</v>
       </c>
       <c r="I8" s="2">
-        <v>2.29872727394104</v>
+        <v>2.3552412986755371</v>
       </c>
       <c r="J8" s="2">
-        <v>2.393510103225708</v>
+        <v>2.4418103694915772</v>
       </c>
       <c r="K8" s="2">
         <v>0</v>
@@ -3474,19 +3474,19 @@
         <v>0</v>
       </c>
       <c r="P8" s="2">
-        <v>3.5506072044372559</v>
+        <v>3.5970621109008789</v>
       </c>
       <c r="Q8" s="2">
         <v>0</v>
       </c>
       <c r="R8" s="2">
-        <v>16.114725112915039</v>
+        <v>16.557954788208008</v>
       </c>
       <c r="S8" s="2">
         <v>0</v>
       </c>
       <c r="T8" s="2">
-        <v>7.6582126617431641</v>
+        <v>7.751190185546875</v>
       </c>
       <c r="U8" s="2">
         <v>0</v>
@@ -3509,22 +3509,22 @@
         <v>20.367532730102539</v>
       </c>
       <c r="E9" s="2">
-        <v>19.02979850769043</v>
+        <v>18.802654266357422</v>
       </c>
       <c r="F9" s="2">
-        <v>17.323177337646484</v>
+        <v>17.153783798217773</v>
       </c>
       <c r="G9" s="2">
-        <v>17.323177337646484</v>
+        <v>17.153783798217773</v>
       </c>
       <c r="H9" s="2">
         <v>2.2978184223175049</v>
       </c>
       <c r="I9" s="2">
-        <v>2.303865909576416</v>
+        <v>2.3605029582977295</v>
       </c>
       <c r="J9" s="2">
-        <v>2.3988547325134277</v>
+        <v>2.4472601413726807</v>
       </c>
       <c r="K9" s="2">
         <v>0</v>
@@ -3542,22 +3542,22 @@
         <v>0</v>
       </c>
       <c r="P9" s="2">
-        <v>2.5500991344451904</v>
+        <v>2.5831165313720703</v>
       </c>
       <c r="Q9" s="2">
-        <v>5.0640344619750977</v>
+        <v>5.8760967254638672</v>
       </c>
       <c r="R9" s="2">
-        <v>19.02979850769043</v>
+        <v>18.802654266357422</v>
       </c>
       <c r="S9" s="2">
         <v>0</v>
       </c>
       <c r="T9" s="2">
-        <v>5.5035552978515625</v>
+        <v>5.5697765350341797</v>
       </c>
       <c r="U9" s="2">
-        <v>11.635647773742676</v>
+        <v>12.156338691711426</v>
       </c>
       <c r="V9" s="2">
         <v>0</v>
@@ -3577,22 +3577,22 @@
         <v>24.781248092651367</v>
       </c>
       <c r="E10" s="2">
-        <v>21.342201232910156</v>
+        <v>20.907466888427734</v>
       </c>
       <c r="F10" s="2">
-        <v>17.888378143310547</v>
+        <v>17.601799011230469</v>
       </c>
       <c r="G10" s="2">
-        <v>17.888378143310547</v>
+        <v>17.601799011230469</v>
       </c>
       <c r="H10" s="2">
         <v>1.7347590923309326</v>
       </c>
       <c r="I10" s="2">
-        <v>1.7393511533737183</v>
+        <v>1.7823628187179565</v>
       </c>
       <c r="J10" s="2">
-        <v>1.8114960193634033</v>
+        <v>1.8482742309570313</v>
       </c>
       <c r="K10" s="2">
         <v>0</v>
@@ -3610,22 +3610,22 @@
         <v>0</v>
       </c>
       <c r="P10" s="2">
-        <v>2.7986464500427246</v>
+        <v>2.8814892768859863</v>
       </c>
       <c r="Q10" s="2">
-        <v>11.490988731384277</v>
+        <v>13.333670616149902</v>
       </c>
       <c r="R10" s="2">
-        <v>21.342201232910156</v>
+        <v>20.907466888427734</v>
       </c>
       <c r="S10" s="2">
         <v>0</v>
       </c>
       <c r="T10" s="2">
-        <v>5.0987820625305176</v>
+        <v>5.2041091918945313</v>
       </c>
       <c r="U10" s="2">
-        <v>26.402877807617188</v>
+        <v>27.584396362304688</v>
       </c>
       <c r="V10" s="2">
         <v>0</v>
@@ -3645,22 +3645,22 @@
         <v>20.247932434082031</v>
       </c>
       <c r="E11" s="2">
-        <v>19.697257995605469</v>
+        <v>19.57783317565918</v>
       </c>
       <c r="F11" s="2">
-        <v>18.07392692565918</v>
+        <v>17.917034149169922</v>
       </c>
       <c r="G11" s="2">
-        <v>18.07392692565918</v>
+        <v>17.917034149169922</v>
       </c>
       <c r="H11" s="2">
         <v>2.789578914642334</v>
       </c>
       <c r="I11" s="2">
-        <v>2.7968838214874268</v>
+        <v>2.8652849197387695</v>
       </c>
       <c r="J11" s="2">
-        <v>2.9115931987762451</v>
+        <v>2.9700307846069336</v>
       </c>
       <c r="K11" s="2">
         <v>0</v>
@@ -3678,22 +3678,22 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
-        <v>13.599834442138672</v>
+        <v>13.933365821838379</v>
       </c>
       <c r="Q11" s="2">
-        <v>2.1205456256866455</v>
+        <v>2.4605934619903565</v>
       </c>
       <c r="R11" s="2">
-        <v>19.697257995605469</v>
+        <v>19.57783317565918</v>
       </c>
       <c r="S11" s="2">
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <v>22.744274139404297</v>
+        <v>23.166378021240234</v>
       </c>
       <c r="U11" s="2">
-        <v>4.8723835945129395</v>
+        <v>5.0904207229614258</v>
       </c>
       <c r="V11" s="2">
         <v>0</v>
@@ -3713,10 +3713,10 @@
         <v>18.470090866088867</v>
       </c>
       <c r="E12" s="2">
-        <v>18.439788818359375</v>
+        <v>18.389963150024414</v>
       </c>
       <c r="F12" s="2">
-        <v>18.353315353393555</v>
+        <v>18.307836532592774</v>
       </c>
       <c r="G12" s="2">
         <v>18.293428421020508</v>
@@ -3725,10 +3725,10 @@
         <v>1.898406982421875</v>
       </c>
       <c r="I12" s="2">
-        <v>1.9034239053726196</v>
+        <v>1.9504127502441406</v>
       </c>
       <c r="J12" s="2">
-        <v>1.9822373390197754</v>
+        <v>2.0224101543426514</v>
       </c>
       <c r="K12" s="2">
         <v>0</v>
@@ -3746,10 +3746,10 @@
         <v>0</v>
       </c>
       <c r="P12" s="2">
-        <v>6.5405168533325195</v>
+        <v>6.6715264320373535</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.62590259313583374</v>
+        <v>0.72627156972885132</v>
       </c>
       <c r="R12" s="2">
         <v>18.293428421020508</v>
@@ -3758,10 +3758,10 @@
         <v>0</v>
       </c>
       <c r="T12" s="2">
-        <v>10.053220748901367</v>
+        <v>10.218766212463379</v>
       </c>
       <c r="U12" s="2">
-        <v>1.4381382465362549</v>
+        <v>1.5024943351745606</v>
       </c>
       <c r="V12" s="2">
         <v>0</v>
@@ -3772,64 +3772,64 @@
         <v>44</v>
       </c>
       <c r="B13" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13" s="2">
-        <v>17.884822845458984</v>
+        <v>30.1993408203125</v>
       </c>
       <c r="D13" s="2">
-        <v>19.097026824951172</v>
+        <v>22.846336364746094</v>
       </c>
       <c r="E13" s="2">
-        <v>19.055629730224609</v>
+        <v>20.703248977661133</v>
       </c>
       <c r="F13" s="2">
-        <v>19.012657165527344</v>
+        <v>18.572671890258789</v>
       </c>
       <c r="G13" s="2">
-        <v>17.884822845458984</v>
+        <v>18.572671890258789</v>
       </c>
       <c r="H13" s="2">
-        <v>0.8641015887260437</v>
+        <v>2.9817616939544678</v>
       </c>
       <c r="I13" s="2">
-        <v>0.86640965938568115</v>
+        <v>3.0625195503234863</v>
       </c>
       <c r="J13" s="2">
-        <v>0.90267860889434815</v>
+        <v>3.1742401123046875</v>
       </c>
       <c r="K13" s="2">
         <v>0</v>
       </c>
       <c r="L13" s="2">
-        <v>0.040168989449739456</v>
+        <v>0</v>
       </c>
       <c r="M13" s="2">
-        <v>-0.53733927011489868</v>
+        <v>-1.0397177934646606</v>
       </c>
       <c r="N13" s="2">
-        <v>17.884822845458984</v>
+        <v>22.846336364746094</v>
       </c>
       <c r="O13" s="2">
         <v>0</v>
       </c>
       <c r="P13" s="2">
-        <v>1.5416826009750366</v>
+        <v>1.8304789066314697</v>
       </c>
       <c r="Q13" s="2">
-        <v>1.656848669052124</v>
+        <v>3.7199921607971192</v>
       </c>
       <c r="R13" s="2">
-        <v>17.884822845458984</v>
+        <v>20.703248977661133</v>
       </c>
       <c r="S13" s="2">
         <v>0</v>
       </c>
       <c r="T13" s="2">
-        <v>3.344538688659668</v>
+        <v>3.9283461570739746</v>
       </c>
       <c r="U13" s="2">
-        <v>3.8069462776184082</v>
+        <v>7.6958365440368652</v>
       </c>
       <c r="V13" s="2">
         <v>0</v>
@@ -3840,67 +3840,67 @@
         <v>45</v>
       </c>
       <c r="B14" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
-        <v>23.573837280273438</v>
+        <v>17.884822845458984</v>
       </c>
       <c r="D14" s="2">
-        <v>22.801759719848633</v>
+        <v>19.097026824951172</v>
       </c>
       <c r="E14" s="2">
-        <v>21.294038772583008</v>
+        <v>19.021995544433594</v>
       </c>
       <c r="F14" s="2">
-        <v>19.267654418945313</v>
+        <v>18.985639572143555</v>
       </c>
       <c r="G14" s="2">
-        <v>19.267654418945313</v>
+        <v>17.884822845458984</v>
       </c>
       <c r="H14" s="2">
-        <v>3.4359700679779053</v>
+        <v>0.8641015887260437</v>
       </c>
       <c r="I14" s="2">
-        <v>3.4449076652526855</v>
+        <v>0.88802939653396607</v>
       </c>
       <c r="J14" s="2">
-        <v>3.585214376449585</v>
+        <v>0.92117851972579956</v>
       </c>
       <c r="K14" s="2">
         <v>0</v>
       </c>
       <c r="L14" s="2">
-        <v>3.5939993858337402</v>
+        <v>0.040168989449739456</v>
       </c>
       <c r="M14" s="2">
-        <v>-1.3353294134140015</v>
+        <v>-0.53733927011489868</v>
       </c>
       <c r="N14" s="2">
-        <v>22.801759719848633</v>
+        <v>17.884822845458984</v>
       </c>
       <c r="O14" s="2">
         <v>0</v>
       </c>
       <c r="P14" s="2">
-        <v>7.571174144744873</v>
+        <v>1.6019192934036255</v>
       </c>
       <c r="Q14" s="2">
-        <v>4.117396354675293</v>
+        <v>1.9225389957427979</v>
       </c>
       <c r="R14" s="2">
-        <v>21.294038772583008</v>
+        <v>17.884822845458984</v>
       </c>
       <c r="S14" s="2">
         <v>0</v>
       </c>
       <c r="T14" s="2">
-        <v>12.33000373840332</v>
+        <v>3.4284920692443848</v>
       </c>
       <c r="U14" s="2">
-        <v>9.4605531692504883</v>
+        <v>3.9773054122924805</v>
       </c>
       <c r="V14" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3911,64 +3911,64 @@
         <v>1</v>
       </c>
       <c r="C15" s="2">
-        <v>30.1993408203125</v>
+        <v>23.573837280273438</v>
       </c>
       <c r="D15" s="2">
-        <v>22.846336364746094</v>
+        <v>22.801759719848633</v>
       </c>
       <c r="E15" s="2">
-        <v>21.588651657104492</v>
+        <v>21.10993766784668</v>
       </c>
       <c r="F15" s="2">
-        <v>19.317661285400391</v>
+        <v>19.124069213867188</v>
       </c>
       <c r="G15" s="2">
-        <v>19.317661285400391</v>
+        <v>19.124069213867188</v>
       </c>
       <c r="H15" s="2">
-        <v>2.9817616939544678</v>
+        <v>3.4359700679779053</v>
       </c>
       <c r="I15" s="2">
-        <v>2.9895541667938233</v>
+        <v>3.5285823345184326</v>
       </c>
       <c r="J15" s="2">
-        <v>3.1119136810302734</v>
+        <v>3.6566627025604248</v>
       </c>
       <c r="K15" s="2">
         <v>0</v>
       </c>
       <c r="L15" s="2">
-        <v>0</v>
+        <v>3.5939993858337402</v>
       </c>
       <c r="M15" s="2">
-        <v>-1.0397177934646606</v>
+        <v>-1.3353294134140015</v>
       </c>
       <c r="N15" s="2">
-        <v>22.846336364746094</v>
+        <v>22.801759719848633</v>
       </c>
       <c r="O15" s="2">
         <v>0</v>
       </c>
       <c r="P15" s="2">
-        <v>1.8054473400115967</v>
+        <v>7.7478733062744141</v>
       </c>
       <c r="Q15" s="2">
-        <v>3.2058982849121094</v>
+        <v>4.7776570320129395</v>
       </c>
       <c r="R15" s="2">
-        <v>21.588651657104492</v>
+        <v>21.10993766784668</v>
       </c>
       <c r="S15" s="2">
         <v>0</v>
       </c>
       <c r="T15" s="2">
-        <v>3.8789291381835938</v>
+        <v>12.552569389343262</v>
       </c>
       <c r="U15" s="2">
-        <v>7.3662018775939942</v>
+        <v>9.8839092254638672</v>
       </c>
       <c r="V15" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3985,22 +3985,22 @@
         <v>27.475223541259766</v>
       </c>
       <c r="E16" s="2">
-        <v>23.602361679077149</v>
+        <v>23.509628295898438</v>
       </c>
       <c r="F16" s="2">
-        <v>19.558908462524414</v>
+        <v>19.485086441040039</v>
       </c>
       <c r="G16" s="2">
-        <v>19.558908462524414</v>
+        <v>19.485086441040039</v>
       </c>
       <c r="H16" s="2">
         <v>7.7605075836181641</v>
       </c>
       <c r="I16" s="2">
-        <v>7.779787540435791</v>
+        <v>7.9600720405578613</v>
       </c>
       <c r="J16" s="2">
-        <v>8.0818710327148438</v>
+        <v>8.2352752685546875</v>
       </c>
       <c r="K16" s="2">
         <v>0</v>
@@ -4018,22 +4018,22 @@
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>23.625207901000977</v>
+        <v>23.963703155517578</v>
       </c>
       <c r="Q16" s="2">
-        <v>4.4317698478698731</v>
+        <v>5.1424431800842285</v>
       </c>
       <c r="R16" s="2">
-        <v>23.602361679077149</v>
+        <v>23.509628295898438</v>
       </c>
       <c r="S16" s="2">
         <v>0</v>
       </c>
       <c r="T16" s="2">
-        <v>32.631767272949219</v>
+        <v>33.053462982177734</v>
       </c>
       <c r="U16" s="2">
-        <v>10.182890892028809</v>
+        <v>10.638571739196777</v>
       </c>
       <c r="V16" s="2">
         <v>0</v>
@@ -4053,22 +4053,22 @@
         <v>28.847429275512695</v>
       </c>
       <c r="E17" s="2">
-        <v>24.574161529541016</v>
+        <v>24.013715744018555</v>
       </c>
       <c r="F17" s="2">
-        <v>20.261716842651367</v>
+        <v>19.874496459960938</v>
       </c>
       <c r="G17" s="2">
-        <v>20.261716842651367</v>
+        <v>19.874496459960938</v>
       </c>
       <c r="H17" s="2">
         <v>1.6044813394546509</v>
       </c>
       <c r="I17" s="2">
-        <v>1.608734130859375</v>
+        <v>1.6485708951950073</v>
       </c>
       <c r="J17" s="2">
-        <v>1.6755548715591431</v>
+        <v>1.7096203565597534</v>
       </c>
       <c r="K17" s="2">
         <v>0</v>
@@ -4086,22 +4086,22 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>17.788810729980469</v>
+        <v>17.862697601318359</v>
       </c>
       <c r="Q17" s="2">
-        <v>12.349308013916016</v>
+        <v>14.329627990722656</v>
       </c>
       <c r="R17" s="2">
-        <v>24.574161529541016</v>
+        <v>24.013715744018555</v>
       </c>
       <c r="S17" s="2">
         <v>0</v>
       </c>
       <c r="T17" s="2">
-        <v>19.443981170654297</v>
+        <v>19.535297393798828</v>
       </c>
       <c r="U17" s="2">
-        <v>28.375041961669922</v>
+        <v>29.644811630249024</v>
       </c>
       <c r="V17" s="2">
         <v>0</v>
@@ -4121,22 +4121,22 @@
         <v>23.07160758972168</v>
       </c>
       <c r="E18" s="2">
-        <v>22.043001174926758</v>
+        <v>21.692031860351563</v>
       </c>
       <c r="F18" s="2">
-        <v>20.684759140014649</v>
+        <v>20.223287582397461</v>
       </c>
       <c r="G18" s="2">
-        <v>20.684759140014649</v>
+        <v>20.223287582397461</v>
       </c>
       <c r="H18" s="2">
         <v>1.4824877977371216</v>
       </c>
       <c r="I18" s="2">
-        <v>1.4864221811294556</v>
+        <v>1.5232763290405274</v>
       </c>
       <c r="J18" s="2">
-        <v>1.5482410192489624</v>
+        <v>1.5797604322433472</v>
       </c>
       <c r="K18" s="2">
         <v>0</v>
@@ -4154,22 +4154,22 @@
         <v>0</v>
       </c>
       <c r="P18" s="2">
-        <v>1.3999004364013672</v>
+        <v>1.4178923368453979</v>
       </c>
       <c r="Q18" s="2">
-        <v>4.144951343536377</v>
+        <v>4.8096308708190918</v>
       </c>
       <c r="R18" s="2">
-        <v>22.043001174926758</v>
+        <v>21.692031860351563</v>
       </c>
       <c r="S18" s="2">
         <v>0</v>
       </c>
       <c r="T18" s="2">
-        <v>3.024561882019043</v>
+        <v>3.0607876777648926</v>
       </c>
       <c r="U18" s="2">
-        <v>9.5238676071166992</v>
+        <v>9.9500570297241211</v>
       </c>
       <c r="V18" s="2">
         <v>0</v>
@@ -4189,10 +4189,10 @@
         <v>21.237567901611328</v>
       </c>
       <c r="E19" s="2">
-        <v>21.083894729614258</v>
+        <v>20.988819122314453</v>
       </c>
       <c r="F19" s="2">
-        <v>20.82861328125</v>
+        <v>20.746059417724609</v>
       </c>
       <c r="G19" s="2">
         <v>20.405284881591797</v>
@@ -4201,10 +4201,10 @@
         <v>1.7534372806549072</v>
       </c>
       <c r="I19" s="2">
-        <v>1.7580786943435669</v>
+        <v>1.8015450239181519</v>
       </c>
       <c r="J19" s="2">
-        <v>1.830985426902771</v>
+        <v>1.8681514263153076</v>
       </c>
       <c r="K19" s="2">
         <v>0</v>
@@ -4222,10 +4222,10 @@
         <v>0</v>
       </c>
       <c r="P19" s="2">
-        <v>4.9063024520874023</v>
+        <v>5.0492429733276367</v>
       </c>
       <c r="Q19" s="2">
-        <v>1.5240592956542969</v>
+        <v>1.7684556245803833</v>
       </c>
       <c r="R19" s="2">
         <v>20.405284881591797</v>
@@ -4234,10 +4234,10 @@
         <v>0</v>
       </c>
       <c r="T19" s="2">
-        <v>8.7677555084228516</v>
+        <v>8.9485607147216797</v>
       </c>
       <c r="U19" s="2">
-        <v>3.5018353462219238</v>
+        <v>3.6585414409637451</v>
       </c>
       <c r="V19" s="2">
         <v>0</v>
@@ -4257,10 +4257,10 @@
         <v>22.671306610107422</v>
       </c>
       <c r="E20" s="2">
-        <v>22.515262603759766</v>
+        <v>22.509096145629883</v>
       </c>
       <c r="F20" s="2">
-        <v>22.354415893554688</v>
+        <v>22.345958709716797</v>
       </c>
       <c r="G20" s="2">
         <v>21.489063262939453</v>
@@ -4269,10 +4269,10 @@
         <v>2.761577844619751</v>
       </c>
       <c r="I20" s="2">
-        <v>2.7688114643096924</v>
+        <v>2.8365466594696045</v>
       </c>
       <c r="J20" s="2">
-        <v>2.8824050426483154</v>
+        <v>2.9402732849121094</v>
       </c>
       <c r="K20" s="2">
         <v>0</v>
@@ -4290,10 +4290,10 @@
         <v>0</v>
       </c>
       <c r="P20" s="2">
-        <v>13.107076644897461</v>
+        <v>13.279899597167969</v>
       </c>
       <c r="Q20" s="2">
-        <v>0.54404634237289429</v>
+        <v>0.63128894567489624</v>
       </c>
       <c r="R20" s="2">
         <v>21.489063262939453</v>
@@ -4302,10 +4302,10 @@
         <v>0</v>
       </c>
       <c r="T20" s="2">
-        <v>17.760456085205078</v>
+        <v>17.978822708129883</v>
       </c>
       <c r="U20" s="2">
-        <v>1.2500569820404053</v>
+        <v>1.3059964179992676</v>
       </c>
       <c r="V20" s="2">
         <v>0</v>
@@ -4325,10 +4325,10 @@
         <v>22.480293273925781</v>
       </c>
       <c r="E21" s="2">
-        <v>22.49610710144043</v>
+        <v>22.532751083374023</v>
       </c>
       <c r="F21" s="2">
-        <v>22.603614807128906</v>
+        <v>22.636785507202148</v>
       </c>
       <c r="G21" s="2">
         <v>22.279586791992188</v>
@@ -4337,10 +4337,10 @@
         <v>1.0774835348129272</v>
       </c>
       <c r="I21" s="2">
-        <v>1.0803548097610474</v>
+        <v>1.1072546243667603</v>
       </c>
       <c r="J21" s="2">
-        <v>1.1254786252975464</v>
+        <v>1.1484918594360352</v>
       </c>
       <c r="K21" s="2">
         <v>0</v>
@@ -4358,10 +4358,10 @@
         <v>0</v>
       </c>
       <c r="P21" s="2">
-        <v>11.277477264404297</v>
+        <v>11.336297988891602</v>
       </c>
       <c r="Q21" s="2">
-        <v>0.58977335691452026</v>
+        <v>0.6843487024307251</v>
       </c>
       <c r="R21" s="2">
         <v>22.279586791992188</v>
@@ -4370,10 +4370,10 @@
         <v>0</v>
       </c>
       <c r="T21" s="2">
-        <v>12.819716453552246</v>
+        <v>12.894399642944336</v>
       </c>
       <c r="U21" s="2">
-        <v>1.3551241159439087</v>
+        <v>1.4157654047012329</v>
       </c>
       <c r="V21" s="2">
         <v>0</v>
@@ -4393,22 +4393,22 @@
         <v>30.89259147644043</v>
       </c>
       <c r="E22" s="2">
-        <v>27.159116744995117</v>
+        <v>26.658615112304688</v>
       </c>
       <c r="F22" s="2">
-        <v>23.102348327636719</v>
+        <v>22.731952667236328</v>
       </c>
       <c r="G22" s="2">
-        <v>23.102348327636719</v>
+        <v>22.731952667236328</v>
       </c>
       <c r="H22" s="2">
         <v>3.1133308410644531</v>
       </c>
       <c r="I22" s="2">
-        <v>3.1214561462402344</v>
+        <v>3.197533130645752</v>
       </c>
       <c r="J22" s="2">
-        <v>3.2490324974060059</v>
+        <v>3.3140106201171875</v>
       </c>
       <c r="K22" s="2">
         <v>0</v>
@@ -4426,22 +4426,22 @@
         <v>0</v>
       </c>
       <c r="P22" s="2">
-        <v>3.3909907341003418</v>
+        <v>3.4340546131134033</v>
       </c>
       <c r="Q22" s="2">
-        <v>7.0988073348999024</v>
+        <v>8.2371625900268555</v>
       </c>
       <c r="R22" s="2">
-        <v>27.159116744995117</v>
+        <v>26.658615112304688</v>
       </c>
       <c r="S22" s="2">
         <v>0</v>
       </c>
       <c r="T22" s="2">
-        <v>7.3215622901916504</v>
+        <v>7.4080705642700195</v>
       </c>
       <c r="U22" s="2">
-        <v>16.310949325561523</v>
+        <v>17.040859222412109</v>
       </c>
       <c r="V22" s="2">
         <v>0</v>
@@ -4452,64 +4452,64 @@
         <v>54</v>
       </c>
       <c r="B23" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="2">
-        <v>23.08891487121582</v>
+        <v>28.985597610473633</v>
       </c>
       <c r="D23" s="2">
-        <v>23.366703033447266</v>
+        <v>26.016490936279297</v>
       </c>
       <c r="E23" s="2">
-        <v>23.404611587524414</v>
+        <v>24.60870361328125</v>
       </c>
       <c r="F23" s="2">
-        <v>23.353071212768555</v>
+        <v>23.246759414672852</v>
       </c>
       <c r="G23" s="2">
-        <v>23.08891487121582</v>
+        <v>23.246759414672852</v>
       </c>
       <c r="H23" s="2">
-        <v>1.8180438280105591</v>
+        <v>1.3418706655502319</v>
       </c>
       <c r="I23" s="2">
-        <v>1.8228522539138794</v>
+        <v>1.3788443803787232</v>
       </c>
       <c r="J23" s="2">
-        <v>1.8983945846557617</v>
+        <v>1.4300507307052612</v>
       </c>
       <c r="K23" s="2">
         <v>0</v>
       </c>
       <c r="L23" s="2">
-        <v>0.45628711581230164</v>
+        <v>0</v>
       </c>
       <c r="M23" s="2">
-        <v>-0.18281856179237366</v>
+        <v>-0.8409494161605835</v>
       </c>
       <c r="N23" s="2">
-        <v>23.08891487121582</v>
+        <v>26.016490936279297</v>
       </c>
       <c r="O23" s="2">
         <v>0</v>
       </c>
       <c r="P23" s="2">
-        <v>2.4035634994506836</v>
+        <v>0.60946601629257202</v>
       </c>
       <c r="Q23" s="2">
-        <v>0.56370842456817627</v>
+        <v>3.0088214874267578</v>
       </c>
       <c r="R23" s="2">
-        <v>23.08891487121582</v>
+        <v>24.60870361328125</v>
       </c>
       <c r="S23" s="2">
         <v>0</v>
       </c>
       <c r="T23" s="2">
-        <v>4.7381362915039063</v>
+        <v>1.3121206760406494</v>
       </c>
       <c r="U23" s="2">
-        <v>1.2952344417572021</v>
+        <v>6.2245821952819824</v>
       </c>
       <c r="V23" s="2">
         <v>0</v>
@@ -4523,61 +4523,61 @@
         <v>3</v>
       </c>
       <c r="C24" s="2">
-        <v>23.520000457763672</v>
+        <v>23.08891487121582</v>
       </c>
       <c r="D24" s="2">
-        <v>23.860641479492188</v>
+        <v>23.366703033447266</v>
       </c>
       <c r="E24" s="2">
-        <v>23.720174789428711</v>
+        <v>23.314310073852539</v>
       </c>
       <c r="F24" s="2">
-        <v>23.550373077392578</v>
+        <v>23.273921966552734</v>
       </c>
       <c r="G24" s="2">
-        <v>23.507095336914063</v>
+        <v>23.08891487121582</v>
       </c>
       <c r="H24" s="2">
-        <v>1.7738965749740601</v>
+        <v>1.8180438280105591</v>
       </c>
       <c r="I24" s="2">
-        <v>1.7785911560058594</v>
+        <v>1.867890477180481</v>
       </c>
       <c r="J24" s="2">
-        <v>1.8523330688476563</v>
+        <v>1.9369018077850342</v>
       </c>
       <c r="K24" s="2">
         <v>0</v>
       </c>
       <c r="L24" s="2">
-        <v>3.2971758842468262</v>
+        <v>0.45628711581230164</v>
       </c>
       <c r="M24" s="2">
-        <v>-0.5881035327911377</v>
+        <v>-0.18281856179237366</v>
       </c>
       <c r="N24" s="2">
-        <v>23.520000457763672</v>
+        <v>23.08891487121582</v>
       </c>
       <c r="O24" s="2">
         <v>0</v>
       </c>
       <c r="P24" s="2">
-        <v>5.3284649848937988</v>
+        <v>2.4901535511016846</v>
       </c>
       <c r="Q24" s="2">
-        <v>1.8133766651153565</v>
+        <v>0.65410399436950684</v>
       </c>
       <c r="R24" s="2">
-        <v>23.520000457763672</v>
+        <v>23.08891487121582</v>
       </c>
       <c r="S24" s="2">
         <v>0</v>
       </c>
       <c r="T24" s="2">
-        <v>7.7642936706542969</v>
+        <v>4.8475685119628906</v>
       </c>
       <c r="U24" s="2">
-        <v>4.1666007041931152</v>
+        <v>1.3531956672668457</v>
       </c>
       <c r="V24" s="2">
         <v>0</v>
@@ -4588,64 +4588,64 @@
         <v>56</v>
       </c>
       <c r="B25" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" s="2">
-        <v>28.985597610473633</v>
+        <v>23.520000457763672</v>
       </c>
       <c r="D25" s="2">
-        <v>26.016490936279297</v>
+        <v>23.860641479492188</v>
       </c>
       <c r="E25" s="2">
-        <v>25.388309478759766</v>
+        <v>23.657814025878906</v>
       </c>
       <c r="F25" s="2">
-        <v>23.901479721069336</v>
+        <v>23.49952507019043</v>
       </c>
       <c r="G25" s="2">
-        <v>23.901479721069336</v>
+        <v>23.486385345458984</v>
       </c>
       <c r="H25" s="2">
-        <v>1.3418706655502319</v>
+        <v>1.7738965749740601</v>
       </c>
       <c r="I25" s="2">
-        <v>1.3454363346099854</v>
+        <v>1.8225553035736084</v>
       </c>
       <c r="J25" s="2">
-        <v>1.4014757871627808</v>
+        <v>1.8899234533309937</v>
       </c>
       <c r="K25" s="2">
         <v>0</v>
       </c>
       <c r="L25" s="2">
-        <v>0</v>
+        <v>3.2971758842468262</v>
       </c>
       <c r="M25" s="2">
-        <v>-0.8409494161605835</v>
+        <v>-0.5881035327911377</v>
       </c>
       <c r="N25" s="2">
-        <v>26.016490936279297</v>
+        <v>23.520000457763672</v>
       </c>
       <c r="O25" s="2">
         <v>0</v>
       </c>
       <c r="P25" s="2">
-        <v>0.60137128829956055</v>
+        <v>5.4193940162658692</v>
       </c>
       <c r="Q25" s="2">
-        <v>2.5930097103118896</v>
+        <v>2.1041674613952637</v>
       </c>
       <c r="R25" s="2">
-        <v>25.388309478759766</v>
+        <v>23.520000457763672</v>
       </c>
       <c r="S25" s="2">
         <v>0</v>
       </c>
       <c r="T25" s="2">
-        <v>1.2959703207015991</v>
+        <v>7.8792562484741211</v>
       </c>
       <c r="U25" s="2">
-        <v>5.9579658508300781</v>
+        <v>4.3530545234680176</v>
       </c>
       <c r="V25" s="2">
         <v>0</v>
@@ -4665,10 +4665,10 @@
         <v>25.706489562988281</v>
       </c>
       <c r="E26" s="2">
-        <v>25.860422134399414</v>
+        <v>25.794523239135742</v>
       </c>
       <c r="F26" s="2">
-        <v>25.961637496948242</v>
+        <v>25.903261184692383</v>
       </c>
       <c r="G26" s="2">
         <v>25.033319473266602</v>
@@ -4677,10 +4677,10 @@
         <v>1.4546895027160645</v>
       </c>
       <c r="I26" s="2">
-        <v>1.4585504531860352</v>
+        <v>1.4947247505187988</v>
       </c>
       <c r="J26" s="2">
-        <v>1.5192286968231201</v>
+        <v>1.5501668453216553</v>
       </c>
       <c r="K26" s="2">
         <v>0</v>
@@ -4698,10 +4698,10 @@
         <v>0</v>
       </c>
       <c r="P26" s="2">
-        <v>3.4249227046966553</v>
+        <v>3.4827728271484375</v>
       </c>
       <c r="Q26" s="2">
-        <v>0.34818267822265625</v>
+        <v>0.40401685237884521</v>
       </c>
       <c r="R26" s="2">
         <v>25.033319473266602</v>
@@ -4710,10 +4710,10 @@
         <v>0</v>
       </c>
       <c r="T26" s="2">
-        <v>4.9794626235961914</v>
+        <v>5.0527057647705078</v>
       </c>
       <c r="U26" s="2">
-        <v>0.80002033710479736</v>
+        <v>0.83582091331481934</v>
       </c>
       <c r="V26" s="2">
         <v>0</v>
@@ -4733,22 +4733,22 @@
         <v>27.460214614868164</v>
       </c>
       <c r="E27" s="2">
-        <v>27.182609558105469</v>
+        <v>27.118217468261719</v>
       </c>
       <c r="F27" s="2">
-        <v>26.370458602905274</v>
+        <v>26.237491607666016</v>
       </c>
       <c r="G27" s="2">
-        <v>26.370458602905274</v>
+        <v>26.237491607666016</v>
       </c>
       <c r="H27" s="2">
         <v>3.6913549900054932</v>
       </c>
       <c r="I27" s="2">
-        <v>3.7009303569793701</v>
+        <v>3.7905797958374023</v>
       </c>
       <c r="J27" s="2">
-        <v>3.8512506484985352</v>
+        <v>3.9277827739715576</v>
       </c>
       <c r="K27" s="2">
         <v>0</v>
@@ -4766,22 +4766,22 @@
         <v>0</v>
       </c>
       <c r="P27" s="2">
-        <v>13.984437942504883</v>
+        <v>14.20643138885498</v>
       </c>
       <c r="Q27" s="2">
-        <v>0.25076732039451599</v>
+        <v>0.29098007082939148</v>
       </c>
       <c r="R27" s="2">
-        <v>27.182609558105469</v>
+        <v>27.118217468261719</v>
       </c>
       <c r="S27" s="2">
         <v>0</v>
       </c>
       <c r="T27" s="2">
-        <v>20.037864685058594</v>
+        <v>20.318199157714844</v>
       </c>
       <c r="U27" s="2">
-        <v>0.57618880271911621</v>
+        <v>0.60197299718856812</v>
       </c>
       <c r="V27" s="2">
         <v>0</v>
@@ -4801,22 +4801,22 @@
         <v>27.974786758422852</v>
       </c>
       <c r="E28" s="2">
-        <v>27.358976364135742</v>
+        <v>27.256763458251953</v>
       </c>
       <c r="F28" s="2">
-        <v>26.71649169921875</v>
+        <v>26.636255264282227</v>
       </c>
       <c r="G28" s="2">
-        <v>26.71649169921875</v>
+        <v>26.636255264282227</v>
       </c>
       <c r="H28" s="2">
         <v>0.90215754508972168</v>
       </c>
       <c r="I28" s="2">
-        <v>0.90456634759902954</v>
+        <v>0.92712974548339844</v>
       </c>
       <c r="J28" s="2">
-        <v>0.94241786003112793</v>
+        <v>0.96172380447387695</v>
       </c>
       <c r="K28" s="2">
         <v>0</v>
@@ -4834,22 +4834,22 @@
         <v>0</v>
       </c>
       <c r="P28" s="2">
-        <v>0.9866936206817627</v>
+        <v>0.99938589334487915</v>
       </c>
       <c r="Q28" s="2">
-        <v>3.3708567619323731</v>
+        <v>3.9114029407501221</v>
       </c>
       <c r="R28" s="2">
-        <v>27.358976364135742</v>
+        <v>27.256763458251953</v>
       </c>
       <c r="S28" s="2">
         <v>0</v>
       </c>
       <c r="T28" s="2">
-        <v>2.1327240467071533</v>
+        <v>2.1583163738250733</v>
       </c>
       <c r="U28" s="2">
-        <v>7.7452268600463867</v>
+        <v>8.091822624206543</v>
       </c>
       <c r="V28" s="2">
         <v>1</v>
@@ -4869,10 +4869,10 @@
         <v>28.952793121337891</v>
       </c>
       <c r="E29" s="2">
-        <v>29.104940414428711</v>
+        <v>29.031343460083008</v>
       </c>
       <c r="F29" s="2">
-        <v>29.191135406494141</v>
+        <v>29.125185012817383</v>
       </c>
       <c r="G29" s="2">
         <v>27.39015007019043</v>
@@ -4881,10 +4881,10 @@
         <v>1.5532145500183105</v>
       </c>
       <c r="I29" s="2">
-        <v>1.5573335886001587</v>
+        <v>1.5959181785583496</v>
       </c>
       <c r="J29" s="2">
-        <v>1.6220545768737793</v>
+        <v>1.6550506353378296</v>
       </c>
       <c r="K29" s="2">
         <v>0</v>
@@ -4902,10 +4902,10 @@
         <v>0</v>
       </c>
       <c r="P29" s="2">
-        <v>2.9402115345001221</v>
+        <v>3.0103855133056641</v>
       </c>
       <c r="Q29" s="2">
-        <v>0.27650368213653565</v>
+        <v>0.32084348797798157</v>
       </c>
       <c r="R29" s="2">
         <v>27.39015007019043</v>
@@ -4914,10 +4914,10 @@
         <v>0</v>
       </c>
       <c r="T29" s="2">
-        <v>4.8595447540283203</v>
+        <v>4.9485855102539063</v>
       </c>
       <c r="U29" s="2">
-        <v>0.63532328605651855</v>
+        <v>0.66375374794006348</v>
       </c>
       <c r="V29" s="2">
         <v>0</v>
@@ -4937,22 +4937,22 @@
         <v>29.355062484741211</v>
       </c>
       <c r="E30" s="2">
-        <v>29.467071533203125</v>
+        <v>29.597591400146484</v>
       </c>
       <c r="F30" s="2">
-        <v>29.695568084716797</v>
+        <v>29.827062606811524</v>
       </c>
       <c r="G30" s="2">
-        <v>29.695568084716797</v>
+        <v>29.827062606811524</v>
       </c>
       <c r="H30" s="2">
         <v>1.1515229940414429</v>
       </c>
       <c r="I30" s="2">
-        <v>1.1545888185501099</v>
+        <v>1.1833148002624512</v>
       </c>
       <c r="J30" s="2">
-        <v>1.2027760744094849</v>
+        <v>1.227350115776062</v>
       </c>
       <c r="K30" s="2">
         <v>0</v>
@@ -4970,22 +4970,22 @@
         <v>0</v>
       </c>
       <c r="P30" s="2">
-        <v>15.223025321960449</v>
+        <v>15.271002769470215</v>
       </c>
       <c r="Q30" s="2">
-        <v>0.15434680879116058</v>
+        <v>0.17909766733646393</v>
       </c>
       <c r="R30" s="2">
-        <v>29.467071533203125</v>
+        <v>29.597591400146484</v>
       </c>
       <c r="S30" s="2">
         <v>0</v>
       </c>
       <c r="T30" s="2">
-        <v>16.435323715209961</v>
+        <v>16.496198654174805</v>
       </c>
       <c r="U30" s="2">
-        <v>0.35464310646057129</v>
+        <v>0.37051323056221008</v>
       </c>
       <c r="V30" s="2">
         <v>0</v>
@@ -5005,22 +5005,22 @@
         <v>32.010368347167969</v>
       </c>
       <c r="E31" s="2">
-        <v>31.759841918945313</v>
+        <v>31.781303405761719</v>
       </c>
       <c r="F31" s="2">
-        <v>31.333070755004883</v>
+        <v>31.355644226074219</v>
       </c>
       <c r="G31" s="2">
-        <v>31.333070755004883</v>
+        <v>31.355644226074219</v>
       </c>
       <c r="H31" s="2">
         <v>3.4333148002624512</v>
       </c>
       <c r="I31" s="2">
-        <v>3.4422454833984375</v>
+        <v>3.5258581638336182</v>
       </c>
       <c r="J31" s="2">
-        <v>3.5824489593505859</v>
+        <v>3.6538434028625488</v>
       </c>
       <c r="K31" s="2">
         <v>0</v>
@@ -5038,22 +5038,22 @@
         <v>0</v>
       </c>
       <c r="P31" s="2">
-        <v>2.2032179832458496</v>
+        <v>2.2335431575775146</v>
       </c>
       <c r="Q31" s="2">
-        <v>0.74716001749038696</v>
+        <v>0.86697375774383545</v>
       </c>
       <c r="R31" s="2">
-        <v>31.759841918945313</v>
+        <v>31.781303405761719</v>
       </c>
       <c r="S31" s="2">
         <v>0</v>
       </c>
       <c r="T31" s="2">
-        <v>4.7337250709533691</v>
+        <v>4.8086299896240234</v>
       </c>
       <c r="U31" s="2">
-        <v>1.7167518138885498</v>
+        <v>1.7935757637023926</v>
       </c>
       <c r="V31" s="2">
         <v>0</v>
@@ -5073,22 +5073,22 @@
         <v>32.506526947021484</v>
       </c>
       <c r="E32" s="2">
-        <v>32.701988220214844</v>
+        <v>32.663913726806641</v>
       </c>
       <c r="F32" s="2">
-        <v>32.886127471923828</v>
+        <v>32.850784301757813</v>
       </c>
       <c r="G32" s="2">
-        <v>32.831272125244141</v>
+        <v>32.817039489746094</v>
       </c>
       <c r="H32" s="2">
         <v>1.6972464323043823</v>
       </c>
       <c r="I32" s="2">
-        <v>1.7017408609390259</v>
+        <v>1.7438398599624634</v>
       </c>
       <c r="J32" s="2">
-        <v>1.7723551988601685</v>
+        <v>1.8083521127700806</v>
       </c>
       <c r="K32" s="2">
         <v>0</v>
@@ -5106,22 +5106,22 @@
         <v>0</v>
       </c>
       <c r="P32" s="2">
-        <v>4.0233664512634277</v>
+        <v>4.0846314430236817</v>
       </c>
       <c r="Q32" s="2">
-        <v>0.080317214131355286</v>
+        <v>0.093196772038936615</v>
       </c>
       <c r="R32" s="2">
-        <v>32.701988220214844</v>
+        <v>32.663913726806641</v>
       </c>
       <c r="S32" s="2">
         <v>0</v>
       </c>
       <c r="T32" s="2">
-        <v>5.6737885475158692</v>
+        <v>5.7513670921325684</v>
       </c>
       <c r="U32" s="2">
-        <v>0.18454508483409882</v>
+        <v>0.19280341267585754</v>
       </c>
       <c r="V32" s="2">
         <v>0</v>
@@ -5141,22 +5141,22 @@
         <v>36.604141235351563</v>
       </c>
       <c r="E33" s="2">
-        <v>35.721961975097656</v>
+        <v>35.563442230224609</v>
       </c>
       <c r="F33" s="2">
-        <v>34.690044403076172</v>
+        <v>34.536983489990234</v>
       </c>
       <c r="G33" s="2">
-        <v>34.690044403076172</v>
+        <v>34.536983489990234</v>
       </c>
       <c r="H33" s="2">
         <v>3.3602819442749024</v>
       </c>
       <c r="I33" s="2">
-        <v>3.3690285682678223</v>
+        <v>3.450925350189209</v>
       </c>
       <c r="J33" s="2">
-        <v>3.5063571929931641</v>
+        <v>3.5762922763824463</v>
       </c>
       <c r="K33" s="2">
         <v>0</v>
@@ -5174,22 +5174,22 @@
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <v>62.195323944091797</v>
+        <v>62.318500518798828</v>
       </c>
       <c r="Q33" s="2">
-        <v>2.0219194889068604</v>
+        <v>2.3461520671844483</v>
       </c>
       <c r="R33" s="2">
-        <v>35.721961975097656</v>
+        <v>35.563442230224609</v>
       </c>
       <c r="S33" s="2">
         <v>0</v>
       </c>
       <c r="T33" s="2">
-        <v>65.091316223144531</v>
+        <v>65.246307373046875</v>
       </c>
       <c r="U33" s="2">
-        <v>4.6457700729370117</v>
+        <v>4.8536663055419922</v>
       </c>
       <c r="V33" s="2">
         <v>0</v>
@@ -5209,22 +5209,22 @@
         <v>35.197097778320313</v>
       </c>
       <c r="E34" s="2">
-        <v>35.275253295898438</v>
+        <v>35.263645172119141</v>
       </c>
       <c r="F34" s="2">
-        <v>35.331844329833984</v>
+        <v>35.308799743652344</v>
       </c>
       <c r="G34" s="2">
-        <v>35.331844329833984</v>
+        <v>35.308799743652344</v>
       </c>
       <c r="H34" s="2">
         <v>2.7869997024536133</v>
       </c>
       <c r="I34" s="2">
-        <v>2.7942979335784912</v>
+        <v>2.8626377582550049</v>
       </c>
       <c r="J34" s="2">
-        <v>2.9089059829711914</v>
+        <v>2.967289924621582</v>
       </c>
       <c r="K34" s="2">
         <v>0</v>
@@ -5242,22 +5242,22 @@
         <v>0</v>
       </c>
       <c r="P34" s="2">
-        <v>2.979482889175415</v>
+        <v>3.0673096179962158</v>
       </c>
       <c r="Q34" s="2">
-        <v>0.32532435655593872</v>
+        <v>0.3774929940700531</v>
       </c>
       <c r="R34" s="2">
-        <v>35.275253295898438</v>
+        <v>35.263645172119141</v>
       </c>
       <c r="S34" s="2">
         <v>0</v>
       </c>
       <c r="T34" s="2">
-        <v>5.348536491394043</v>
+        <v>5.4593148231506348</v>
       </c>
       <c r="U34" s="2">
-        <v>0.74749875068664551</v>
+        <v>0.78094905614852905</v>
       </c>
       <c r="V34" s="2">
         <v>0</v>
@@ -5277,22 +5277,22 @@
         <v>37.775814056396484</v>
       </c>
       <c r="E35" s="2">
-        <v>37.467479705810547</v>
+        <v>37.332427978515625</v>
       </c>
       <c r="F35" s="2">
-        <v>36.946628570556641</v>
+        <v>36.76470947265625</v>
       </c>
       <c r="G35" s="2">
-        <v>36.946628570556641</v>
+        <v>36.76470947265625</v>
       </c>
       <c r="H35" s="2">
         <v>0.26343199610710144</v>
       </c>
       <c r="I35" s="2">
-        <v>0.26413977146148682</v>
+        <v>0.27077224850654602</v>
       </c>
       <c r="J35" s="2">
-        <v>0.27526739239692688</v>
+        <v>0.28094503283500671</v>
       </c>
       <c r="K35" s="2">
         <v>0</v>
@@ -5310,22 +5310,22 @@
         <v>0</v>
       </c>
       <c r="P35" s="2">
-        <v>0.12676049768924713</v>
+        <v>0.12845955789089203</v>
       </c>
       <c r="Q35" s="2">
-        <v>2.2025189399719238</v>
+        <v>2.5557119846343994</v>
       </c>
       <c r="R35" s="2">
-        <v>37.467479705810547</v>
+        <v>37.332427978515625</v>
       </c>
       <c r="S35" s="2">
         <v>0</v>
       </c>
       <c r="T35" s="2">
-        <v>0.27348038554191589</v>
+        <v>0.2768833339214325</v>
       </c>
       <c r="U35" s="2">
-        <v>5.0607342720031738</v>
+        <v>5.2871999740600586</v>
       </c>
       <c r="V35" s="2">
         <v>1</v>
@@ -5345,22 +5345,22 @@
         <v>38.860160827636719</v>
       </c>
       <c r="E36" s="2">
-        <v>38.666847229003906</v>
+        <v>38.473709106445313</v>
       </c>
       <c r="F36" s="2">
-        <v>38.296337127685547</v>
+        <v>38.139186859130859</v>
       </c>
       <c r="G36" s="2">
-        <v>38.296337127685547</v>
+        <v>38.139186859130859</v>
       </c>
       <c r="H36" s="2">
         <v>0.71748131513595581</v>
       </c>
       <c r="I36" s="2">
-        <v>0.71939992904663086</v>
+        <v>0.73737931251525879</v>
       </c>
       <c r="J36" s="2">
-        <v>0.74956214427947998</v>
+        <v>0.76494818925857544</v>
       </c>
       <c r="K36" s="2">
         <v>0</v>
@@ -5378,22 +5378,22 @@
         <v>0</v>
       </c>
       <c r="P36" s="2">
-        <v>0.56380605697631836</v>
+        <v>0.5702400803565979</v>
       </c>
       <c r="Q36" s="2">
-        <v>1.0013796091079712</v>
+        <v>1.1619595289230347</v>
       </c>
       <c r="R36" s="2">
-        <v>38.666847229003906</v>
+        <v>38.473709106445313</v>
       </c>
       <c r="S36" s="2">
         <v>0</v>
       </c>
       <c r="T36" s="2">
-        <v>1.227403998374939</v>
+        <v>1.2407059669494629</v>
       </c>
       <c r="U36" s="2">
-        <v>2.300872802734375</v>
+        <v>2.4038360118865967</v>
       </c>
       <c r="V36" s="2">
         <v>0</v>
@@ -5413,22 +5413,22 @@
         <v>41.151679992675781</v>
       </c>
       <c r="E37" s="2">
-        <v>39.780727386474609</v>
+        <v>39.647865295410156</v>
       </c>
       <c r="F37" s="2">
-        <v>38.526203155517578</v>
+        <v>38.450096130371094</v>
       </c>
       <c r="G37" s="2">
-        <v>38.526203155517578</v>
+        <v>38.450096130371094</v>
       </c>
       <c r="H37" s="2">
         <v>1.8510552644729614</v>
       </c>
       <c r="I37" s="2">
-        <v>1.8559492826461792</v>
+        <v>1.9017889499664307</v>
       </c>
       <c r="J37" s="2">
-        <v>1.9328348636627197</v>
+        <v>1.972027063369751</v>
       </c>
       <c r="K37" s="2">
         <v>0</v>
@@ -5446,22 +5446,22 @@
         <v>0</v>
       </c>
       <c r="P37" s="2">
-        <v>3.6911201477050781</v>
+        <v>3.7526285648345947</v>
       </c>
       <c r="Q37" s="2">
-        <v>3.0927493572235108</v>
+        <v>3.5886988639831543</v>
       </c>
       <c r="R37" s="2">
-        <v>39.780727386474609</v>
+        <v>39.647865295410156</v>
       </c>
       <c r="S37" s="2">
         <v>0</v>
       </c>
       <c r="T37" s="2">
-        <v>5.3476452827453613</v>
+        <v>5.425480842590332</v>
       </c>
       <c r="U37" s="2">
-        <v>7.1062188148498535</v>
+        <v>7.4242191314697266</v>
       </c>
       <c r="V37" s="2">
         <v>0</v>
@@ -5475,61 +5475,61 @@
         <v>1</v>
       </c>
       <c r="C38" s="2">
-        <v>48.211658477783203</v>
+        <v>47.321636199951172</v>
       </c>
       <c r="D38" s="2">
-        <v>46.126636505126953</v>
+        <v>46.450332641601563</v>
       </c>
       <c r="E38" s="2">
-        <v>45.362030029296875</v>
+        <v>45.612285614013672</v>
       </c>
       <c r="F38" s="2">
-        <v>44.914016723632813</v>
+        <v>44.992530822753906</v>
       </c>
       <c r="G38" s="2">
-        <v>44.914016723632813</v>
+        <v>44.992530822753906</v>
       </c>
       <c r="H38" s="2">
-        <v>2.0536274909973145</v>
+        <v>2.2315900325775146</v>
       </c>
       <c r="I38" s="2">
-        <v>2.0590455532073975</v>
+        <v>2.2925102710723877</v>
       </c>
       <c r="J38" s="2">
-        <v>2.1441617012023926</v>
+        <v>2.3768291473388672</v>
       </c>
       <c r="K38" s="2">
         <v>0</v>
       </c>
       <c r="L38" s="2">
-        <v>1.1735610961914063</v>
+        <v>0.11501646786928177</v>
       </c>
       <c r="M38" s="2">
-        <v>-0.31837686896324158</v>
+        <v>-0.57308226823806763</v>
       </c>
       <c r="N38" s="2">
-        <v>46.126636505126953</v>
+        <v>46.450332641601563</v>
       </c>
       <c r="O38" s="2">
         <v>0</v>
       </c>
       <c r="P38" s="2">
-        <v>2.8712136745452881</v>
+        <v>1.3056190013885498</v>
       </c>
       <c r="Q38" s="2">
-        <v>0.98169320821762085</v>
+        <v>2.0504231452941895</v>
       </c>
       <c r="R38" s="2">
-        <v>45.362030029296875</v>
+        <v>45.612285614013672</v>
       </c>
       <c r="S38" s="2">
         <v>0</v>
       </c>
       <c r="T38" s="2">
-        <v>4.9083013534545899</v>
+        <v>2.6823012828826904</v>
       </c>
       <c r="U38" s="2">
-        <v>2.2556393146514893</v>
+        <v>4.2418694496154785</v>
       </c>
       <c r="V38" s="2">
         <v>0</v>
@@ -5543,61 +5543,61 @@
         <v>1</v>
       </c>
       <c r="C39" s="2">
-        <v>47.321636199951172</v>
+        <v>48.211658477783203</v>
       </c>
       <c r="D39" s="2">
-        <v>46.450332641601563</v>
+        <v>46.126636505126953</v>
       </c>
       <c r="E39" s="2">
-        <v>45.747444152832031</v>
+        <v>45.675785064697266</v>
       </c>
       <c r="F39" s="2">
-        <v>45.085468292236328</v>
+        <v>45.188304901123047</v>
       </c>
       <c r="G39" s="2">
-        <v>45.085468292236328</v>
+        <v>45.188304901123047</v>
       </c>
       <c r="H39" s="2">
-        <v>2.2315900325775146</v>
+        <v>2.0536274909973145</v>
       </c>
       <c r="I39" s="2">
-        <v>2.2374672889709473</v>
+        <v>2.1097939014434815</v>
       </c>
       <c r="J39" s="2">
-        <v>2.3297841548919678</v>
+        <v>2.1875436305999756</v>
       </c>
       <c r="K39" s="2">
         <v>0</v>
       </c>
       <c r="L39" s="2">
-        <v>0.11501646786928177</v>
+        <v>1.1735610961914063</v>
       </c>
       <c r="M39" s="2">
-        <v>-0.57308226823806763</v>
+        <v>-0.31837686896324158</v>
       </c>
       <c r="N39" s="2">
-        <v>46.450332641601563</v>
+        <v>46.126636505126953</v>
       </c>
       <c r="O39" s="2">
         <v>0</v>
       </c>
       <c r="P39" s="2">
-        <v>1.2540650367736816</v>
+        <v>2.9453613758087158</v>
       </c>
       <c r="Q39" s="2">
-        <v>1.7670596837997437</v>
+        <v>1.1391164064407349</v>
       </c>
       <c r="R39" s="2">
-        <v>45.747444152832031</v>
+        <v>45.675785064697266</v>
       </c>
       <c r="S39" s="2">
         <v>0</v>
       </c>
       <c r="T39" s="2">
-        <v>2.6174581050872803</v>
+        <v>5.0023350715637207</v>
       </c>
       <c r="U39" s="2">
-        <v>4.060178279876709</v>
+        <v>2.3565783500671387</v>
       </c>
       <c r="V39" s="2">
         <v>0</v>
@@ -5617,22 +5617,22 @@
         <v>50.5023193359375</v>
       </c>
       <c r="E40" s="2">
-        <v>49.833286285400391</v>
+        <v>49.534835815429688</v>
       </c>
       <c r="F40" s="2">
-        <v>48.988327026367188</v>
+        <v>48.752876281738281</v>
       </c>
       <c r="G40" s="2">
-        <v>48.988327026367188</v>
+        <v>48.752876281738281</v>
       </c>
       <c r="H40" s="2">
         <v>2.9550719261169434</v>
       </c>
       <c r="I40" s="2">
-        <v>2.9627969264984131</v>
+        <v>3.0351288318634033</v>
       </c>
       <c r="J40" s="2">
-        <v>3.0840957164764404</v>
+        <v>3.1458826065063477</v>
       </c>
       <c r="K40" s="2">
         <v>0</v>
@@ -5650,22 +5650,22 @@
         <v>0</v>
       </c>
       <c r="P40" s="2">
-        <v>21.232250213623047</v>
+        <v>21.289615631103516</v>
       </c>
       <c r="Q40" s="2">
-        <v>2.406200647354126</v>
+        <v>2.7920560836791992</v>
       </c>
       <c r="R40" s="2">
-        <v>49.833286285400391</v>
+        <v>49.534835815429688</v>
       </c>
       <c r="S40" s="2">
         <v>0</v>
       </c>
       <c r="T40" s="2">
-        <v>22.659465789794922</v>
+        <v>22.731925964355469</v>
       </c>
       <c r="U40" s="2">
-        <v>5.5287342071533203</v>
+        <v>5.7761430740356445</v>
       </c>
       <c r="V40" s="2">
         <v>1</v>
@@ -5685,22 +5685,22 @@
         <v>50.261219024658203</v>
       </c>
       <c r="E41" s="2">
-        <v>50.390838623046875</v>
+        <v>50.496246337890625</v>
       </c>
       <c r="F41" s="2">
-        <v>50.701709747314453</v>
+        <v>50.789035797119141</v>
       </c>
       <c r="G41" s="2">
-        <v>50.701709747314453</v>
+        <v>50.789035797119141</v>
       </c>
       <c r="H41" s="2">
         <v>1.2299784421920776</v>
       </c>
       <c r="I41" s="2">
-        <v>1.233251690864563</v>
+        <v>1.2639086246490479</v>
       </c>
       <c r="J41" s="2">
-        <v>1.2846781015396118</v>
+        <v>1.3109031915664673</v>
       </c>
       <c r="K41" s="2">
         <v>0</v>
@@ -5718,22 +5718,22 @@
         <v>0</v>
       </c>
       <c r="P41" s="2">
-        <v>0.77300810813903809</v>
+        <v>0.78292030096054077</v>
       </c>
       <c r="Q41" s="2">
-        <v>0.096868947148323059</v>
+        <v>0.11240273714065552</v>
       </c>
       <c r="R41" s="2">
-        <v>50.390838623046875</v>
+        <v>50.496246337890625</v>
       </c>
       <c r="S41" s="2">
         <v>0</v>
       </c>
       <c r="T41" s="2">
-        <v>1.6706951856613159</v>
+        <v>1.6906771659851074</v>
       </c>
       <c r="U41" s="2">
-        <v>0.22257606685161591</v>
+        <v>0.23253625631332397</v>
       </c>
       <c r="V41" s="2">
         <v>0</v>
@@ -5753,10 +5753,10 @@
         <v>59.646335601806641</v>
       </c>
       <c r="E42" s="2">
-        <v>59.743328094482422</v>
+        <v>59.817584991455078</v>
       </c>
       <c r="F42" s="2">
-        <v>60.099044799804688</v>
+        <v>60.173206329345703</v>
       </c>
       <c r="G42" s="2">
         <v>58.708148956298828</v>
@@ -5765,10 +5765,10 @@
         <v>1.922600269317627</v>
       </c>
       <c r="I42" s="2">
-        <v>1.9276797771453857</v>
+        <v>1.975255012512207</v>
       </c>
       <c r="J42" s="2">
-        <v>2.0074760913848877</v>
+        <v>2.0481503009796143</v>
       </c>
       <c r="K42" s="2">
         <v>0</v>
@@ -5786,10 +5786,10 @@
         <v>0</v>
       </c>
       <c r="P42" s="2">
-        <v>6.7217693328857422</v>
+        <v>6.7473130226135254</v>
       </c>
       <c r="Q42" s="2">
-        <v>0.87060195207595825</v>
+        <v>1.0102106332778931</v>
       </c>
       <c r="R42" s="2">
         <v>58.708148956298828</v>
@@ -5798,10 +5798,10 @@
         <v>0</v>
       </c>
       <c r="T42" s="2">
-        <v>7.3928213119506836</v>
+        <v>7.4253077507019043</v>
       </c>
       <c r="U42" s="2">
-        <v>2.0003848075866699</v>
+        <v>2.0899012088775635</v>
       </c>
       <c r="V42" s="2">
         <v>1</v>
@@ -5821,22 +5821,22 @@
         <v>70.389595031738281</v>
       </c>
       <c r="E43" s="2">
-        <v>68.067916870117188</v>
+        <v>67.630302429199219</v>
       </c>
       <c r="F43" s="2">
-        <v>65.76434326171875</v>
+        <v>65.465072631835938</v>
       </c>
       <c r="G43" s="2">
-        <v>65.76434326171875</v>
+        <v>65.465072631835938</v>
       </c>
       <c r="H43" s="2">
         <v>0.70774167776107788</v>
       </c>
       <c r="I43" s="2">
-        <v>0.70963507890701294</v>
+        <v>0.72737187147140503</v>
       </c>
       <c r="J43" s="2">
-        <v>0.73939061164855957</v>
+        <v>0.75456911325454712</v>
       </c>
       <c r="K43" s="2">
         <v>0</v>
@@ -5854,22 +5854,22 @@
         <v>0</v>
       </c>
       <c r="P43" s="2">
-        <v>0.33011433482170105</v>
+        <v>0.33433330059051514</v>
       </c>
       <c r="Q43" s="2">
-        <v>3.7623240947723389</v>
+        <v>4.3656458854675293</v>
       </c>
       <c r="R43" s="2">
-        <v>68.067916870117188</v>
+        <v>67.630302429199219</v>
       </c>
       <c r="S43" s="2">
         <v>0</v>
       </c>
       <c r="T43" s="2">
-        <v>0.71392130851745605</v>
+        <v>0.72244465351104736</v>
       </c>
       <c r="U43" s="2">
-        <v>8.6447019577026367</v>
+        <v>9.0315494537353516</v>
       </c>
       <c r="V43" s="2">
         <v>0</v>
@@ -5889,22 +5889,22 @@
         <v>67.48773193359375</v>
       </c>
       <c r="E44" s="2">
-        <v>66.719528198242188</v>
+        <v>66.518142700195313</v>
       </c>
       <c r="F44" s="2">
-        <v>65.958328247070313</v>
+        <v>65.812202453613281</v>
       </c>
       <c r="G44" s="2">
-        <v>65.958328247070313</v>
+        <v>65.812202453613281</v>
       </c>
       <c r="H44" s="2">
         <v>1.3864593505859375</v>
       </c>
       <c r="I44" s="2">
-        <v>1.3901424407958984</v>
+        <v>1.4246439933776856</v>
       </c>
       <c r="J44" s="2">
-        <v>1.4480159282684326</v>
+        <v>1.4775255918502808</v>
       </c>
       <c r="K44" s="2">
         <v>0</v>
@@ -5922,22 +5922,22 @@
         <v>0</v>
       </c>
       <c r="P44" s="2">
-        <v>0.4866364598274231</v>
+        <v>0.49293828010559082</v>
       </c>
       <c r="Q44" s="2">
-        <v>1.4056799411773682</v>
+        <v>1.6310930252075195</v>
       </c>
       <c r="R44" s="2">
-        <v>66.719528198242188</v>
+        <v>66.518142700195313</v>
       </c>
       <c r="S44" s="2">
         <v>0</v>
       </c>
       <c r="T44" s="2">
-        <v>1.051026463508606</v>
+        <v>1.0636987686157227</v>
       </c>
       <c r="U44" s="2">
-        <v>3.2298350334167481</v>
+        <v>3.3743689060211182</v>
       </c>
       <c r="V44" s="2">
         <v>1</v>
@@ -5957,22 +5957,22 @@
         <v>65.348159790039063</v>
       </c>
       <c r="E45" s="2">
-        <v>65.954849243164063</v>
+        <v>66.0341796875</v>
       </c>
       <c r="F45" s="2">
-        <v>66.768684387207031</v>
+        <v>66.834907531738281</v>
       </c>
       <c r="G45" s="2">
-        <v>66.227127075195313</v>
+        <v>66.235137939453125</v>
       </c>
       <c r="H45" s="2">
         <v>1.879230260848999</v>
       </c>
       <c r="I45" s="2">
-        <v>1.8841978311538696</v>
+        <v>1.9307215213775635</v>
       </c>
       <c r="J45" s="2">
-        <v>1.9622311592102051</v>
+        <v>2.0020067691802979</v>
       </c>
       <c r="K45" s="2">
         <v>0</v>
@@ -5990,22 +5990,22 @@
         <v>0</v>
       </c>
       <c r="P45" s="2">
-        <v>7.1902790069580078</v>
+        <v>7.2188591957092285</v>
       </c>
       <c r="Q45" s="2">
-        <v>0.0086023034527897835</v>
+        <v>0.0099817579612135887</v>
       </c>
       <c r="R45" s="2">
-        <v>65.954849243164063</v>
+        <v>66.006317138671875</v>
       </c>
       <c r="S45" s="2">
         <v>0</v>
       </c>
       <c r="T45" s="2">
-        <v>7.9046025276184082</v>
+        <v>7.9406166076660156</v>
       </c>
       <c r="U45" s="2">
-        <v>0.019765537232160568</v>
+        <v>0.020650038495659828</v>
       </c>
       <c r="V45" s="2">
         <v>0</v>
@@ -6025,22 +6025,22 @@
         <v>83.753578186035156</v>
       </c>
       <c r="E46" s="2">
-        <v>82.537696838378906</v>
+        <v>82.392471313476563</v>
       </c>
       <c r="F46" s="2">
-        <v>81.006446838378906</v>
+        <v>80.940452575683594</v>
       </c>
       <c r="G46" s="2">
-        <v>81.006446838378906</v>
+        <v>80.940452575683594</v>
       </c>
       <c r="H46" s="2">
         <v>4.0880637168884277</v>
       </c>
       <c r="I46" s="2">
-        <v>4.0986251831054688</v>
+        <v>4.1974864006042481</v>
       </c>
       <c r="J46" s="2">
-        <v>4.2643814086914063</v>
+        <v>4.3487539291381836</v>
       </c>
       <c r="K46" s="2">
         <v>0</v>
@@ -6058,22 +6058,22 @@
         <v>0</v>
       </c>
       <c r="P46" s="2">
-        <v>1.4657578468322754</v>
+        <v>1.4844467639923096</v>
       </c>
       <c r="Q46" s="2">
-        <v>1.5694382190704346</v>
+        <v>1.8211113214492798</v>
       </c>
       <c r="R46" s="2">
-        <v>82.537696838378906</v>
+        <v>82.392471313476563</v>
       </c>
       <c r="S46" s="2">
         <v>0</v>
       </c>
       <c r="T46" s="2">
-        <v>3.1614346504211426</v>
+        <v>3.1988444328308105</v>
       </c>
       <c r="U46" s="2">
-        <v>3.6061027050018311</v>
+        <v>3.7674746513366699</v>
       </c>
       <c r="V46" s="2">
         <v>0</v>
@@ -6093,22 +6093,22 @@
         <v>89.2027587890625</v>
       </c>
       <c r="E47" s="2">
-        <v>85.987754821777344</v>
+        <v>85.693046569824219</v>
       </c>
       <c r="F47" s="2">
-        <v>82.659873962402344</v>
+        <v>82.49462890625</v>
       </c>
       <c r="G47" s="2">
-        <v>82.659873962402344</v>
+        <v>82.49462890625</v>
       </c>
       <c r="H47" s="2">
         <v>7.6652612686157227</v>
       </c>
       <c r="I47" s="2">
-        <v>7.6843242645263672</v>
+        <v>7.8625850677490234</v>
       </c>
       <c r="J47" s="2">
-        <v>7.9830231666564941</v>
+        <v>8.1347169876098633</v>
       </c>
       <c r="K47" s="2">
         <v>0</v>
@@ -6126,22 +6126,22 @@
         <v>0</v>
       </c>
       <c r="P47" s="2">
-        <v>30.911529541015625</v>
+        <v>31.026357650756836</v>
       </c>
       <c r="Q47" s="2">
-        <v>3.0956614017486572</v>
+        <v>3.5920777320861817</v>
       </c>
       <c r="R47" s="2">
-        <v>85.987754821777344</v>
+        <v>85.693046569824219</v>
       </c>
       <c r="S47" s="2">
         <v>0</v>
       </c>
       <c r="T47" s="2">
-        <v>34.089584350585938</v>
+        <v>34.23486328125</v>
       </c>
       <c r="U47" s="2">
-        <v>7.112910270690918</v>
+        <v>7.4312100410461426</v>
       </c>
       <c r="V47" s="2">
         <v>0</v>
@@ -6199,19 +6199,19 @@
         <v>13.444534301757813</v>
       </c>
       <c r="E2" s="2">
-        <v>7.997016429901123</v>
+        <v>7.0417094230651855</v>
       </c>
       <c r="F2" s="2">
-        <v>1.9058444499969482</v>
+        <v>1.1889625787734985</v>
       </c>
       <c r="G2" s="2">
-        <v>1.9058444499969482</v>
+        <v>1.1889625787734985</v>
       </c>
       <c r="H2" s="2">
-        <v>28.659156799316406</v>
+        <v>28.97459602355957</v>
       </c>
       <c r="I2" s="2">
-        <v>57.303966522216797</v>
+        <v>59.868293762207031</v>
       </c>
     </row>
     <row r="3">
@@ -6228,19 +6228,19 @@
         <v>14.296926498413086</v>
       </c>
       <c r="E3" s="2">
-        <v>9.0769309997558594</v>
+        <v>8.385279655456543</v>
       </c>
       <c r="F3" s="2">
-        <v>3.4344329833984375</v>
+        <v>2.9253649711608887</v>
       </c>
       <c r="G3" s="2">
-        <v>3.4344329833984375</v>
+        <v>2.9253649711608887</v>
       </c>
       <c r="H3" s="2">
-        <v>27.667943954467773</v>
+        <v>28.14610481262207</v>
       </c>
       <c r="I3" s="2">
-        <v>52.961891174316406</v>
+        <v>55.331912994384766</v>
       </c>
     </row>
     <row r="4">
@@ -6257,19 +6257,19 @@
         <v>14.114684104919434</v>
       </c>
       <c r="E4" s="2">
-        <v>11.191521644592285</v>
+        <v>10.987530708312988</v>
       </c>
       <c r="F4" s="2">
-        <v>7.7347092628479004</v>
+        <v>7.5367732048034668</v>
       </c>
       <c r="G4" s="2">
-        <v>7.7347092628479004</v>
+        <v>7.5367732048034668</v>
       </c>
       <c r="H4" s="2">
-        <v>39.587791442871094</v>
+        <v>40.338081359863281</v>
       </c>
       <c r="I4" s="2">
-        <v>7.6455507278442383</v>
+        <v>7.9876861572265625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>